<commit_message>
Add HCM district map labels, reference points, itinerary overlay, card detail dialog, and UI polish
- map_builder: add 19 HCM district badge labels (orange for itinerary districts D1/D2/D3/D5/D9, grey for others)
- map_builder: add reference point markers (beaches, markets, landmarks, airports)
- map_builder: add optional itinerary stops layer; multi-city Vietnam center view
- app.py: card detail dialog via @st.dialog with photo, amenities, remarks, links
- app.py: session-state tab navigation to prevent tab reset on rerun
- app.py: larger card fonts, consistent card heights, dark action buttons
- itinerary_stops.py: trip itinerary stops data file
</commit_message>
<xml_diff>
--- a/stays.xlsx
+++ b/stays.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dika\belajar\Viet\stay_picker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E7E6978-00A8-4F5B-9F4B-845BA17AA80A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E8DE25-939B-4751-B0A4-DE679F4711A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stays" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="160">
   <si>
     <t>FIXED: Sheet renamed to Stays. Distance categories corrected. Dana Home MT price fixed to 1600000. Yellow cells = corrected values.</t>
   </si>
@@ -321,6 +321,195 @@
   </si>
   <si>
     <t>https://google.com/maps/place/Mercury+Beach+House/@16.0884991,108.2460601,17z/data=!4m10!3m9!1s0x314217f213c3031f:0xc3fa594a2c3558c1!5m2!4m1!1i2!8m2!3d16.0884991!4d108.248635!15sCjRNZXJjdXJ5IEJlYWNoIHdpdGggMkJScy0zIEJlZHMtUE9PTCAxMG0gdG8gdGhlIGJlYWNokgEFaG90ZWzgAQA!16s%2Fg%2F11jsp4x6y6?entry=tts&amp;g_ep=EgoyMDI2MDUwMi4wIPu8ASoASAFQAw%3D%3D&amp;skid=1ede066e-c2ca-421e-b8be-8fb412b82088</t>
+  </si>
+  <si>
+    <t>2BR Apm w/ Projector -Dragon Bridge</t>
+  </si>
+  <si>
+    <t>Ada proyektor gibli,Vibes rumah, deket Han River</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1524510118720108105?unique_share_id=a5059c79-d31c-42c2-9a53-23529c164511&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778748636_P3msXIUemTpi-RzF&amp;check_in=2026-07-29&amp;guests=5&amp;adults=5&amp;check_out=2026-08-01</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1523837873251712139/original/15208731-da9a-4e39-beb5-2113a26d0d9d.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/M%E1%BB%99c+Garden+Coffee/@16.059231,108.2301389,19.46z/data=!4m6!3m5!1s0x314219d054c5fd5d:0x62af41bd603ee1ee!8m2!3d16.0596904!4d108.2305975!16s%2Fg%2F11h_v712xq?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>Beachfront - ocean view - 40st floor -nice balcony</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1568686818040745133?unique_share_id=5a957173-1bcd-4f21-b453-2ec722823a4d&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778748939_P3AvY_N8AaLyyzcC&amp;guests=5&amp;adults=5&amp;check_in=2026-07-29&amp;check_out=2026-08-01</t>
+  </si>
+  <si>
+    <t>Ocean view, ada balcon, 70m ke pantai, internet 500 mbps</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1568686818040745133/original/a14fe56c-6d74-4c44-8970-bb349b6b8c13.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/M%C6%B0%E1%BB%9Dng+Thanh+Luxury+Da+Nang+Hotel/@16.0537937,108.2471881,19.73z/data=!4m17!1m7!3m6!1s0x31421778a62cf453:0xb8711a06c7374f9f!2sH2T+Fashion!8m2!3d16.0539812!4d108.2477636!16s%2Fg%2F11stxv7dzj!3m8!1s0x3142177a5081b45b:0x1dba027958889476!5m2!4m1!1i2!8m2!3d16.0537195!4d108.2473341!16s%2Fg%2F11g7316zh1?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>Beachside Duplex • Cozy &amp; Modern • 20% Promo | 102</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1312945023723633727?unique_share_id=a57174dd-3f19-4544-af0a-6a5f17561175&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778749346_P3T20WqcKLFJ-1xy</t>
+  </si>
+  <si>
+    <t>Duplex alias 2 lantai, vibes kosan, 700m ke My Khe Beach, di ground floor, internet 1 Gbps</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-U3RheVN1cHBseUxpc3Rpbmc6MTMxMjk0NTAyMzcyMzYzMzcyNw==/original/a7756e09-0c04-4a76-b477-7fa4dc9786ba.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Doll+Coffee/@16.0552432,108.2410491,21z/data=!4m6!3m5!1s0x3142177c48db3031:0xe3d41529460b71c2!8m2!3d16.0552836!4d108.2412094!16s%2Fg%2F11csq86xyk?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Namto House Near Han Market &amp; Pink Church, 4B
+</t>
+  </si>
+  <si>
+    <t>Rumah, free laundry, bisa req daily cleaning free, bandara 8 menit, pantai 10 menit</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/31482377?unique_share_id=87d22d37-5e24-4620-88fe-bac8a9899616&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778749751_P3-pdNc5YdeFLcg_&amp;check_in=2026-07-29&amp;guests=5&amp;adults=5&amp;check_out=2026-08-01</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-31482377/original/940ae76f-c863-434e-a3e8-cd98f1437fad.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/16.067606,+108.221294?entry=tts&amp;g_ep=EgoyMDI2MDUxMS4wIPu8ASoASAFQAw%3D%3D&amp;skid=9211b561-fba9-49b4-acf8-1e46f1c86088</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Peaceful] 3BR Apart |Garden | Library |Laundry
+</t>
+  </si>
+  <si>
+    <t>Lt 3 Rumah, self check in, ada taman &amp; perpus</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1183818880434998490?unique_share_id=e42050f6-d89b-456e-928c-5a3fe7581e58&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778750162_P31K_RdHMuesPpS3</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1183818880434998490/original/0ebe07cd-5402-4fc6-b2e4-5c55a11869ce.png?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/The+Wooden+Page/@16.0816664,108.2334076,19.91z/data=!4m17!1m7!3m6!1s0x3142192ea7af17a7:0xc89a2c1fa256fb94!2zUXXDoW4gTeG6uSBLZW4!8m2!3d16.0822394!4d108.2332973!16s%2Fg%2F11ststlgnz!3m8!1s0x31421793e1758355:0x8ed7d69dd01fc78b!5m2!4m1!1i2!8m2!3d16.081863!4d108.2338518!16s%2Fg%2F11tn6kcvmm?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beautiful Prime Location Apartment With Ocean View
+</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1598177947715448803/original/a81872e7-6308-46c4-8b0c-c2a38730ae3c.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>Vibes Jardin, deket pantai</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1598177947715448803?unique_share_id=9f2dbfff-682b-41b4-8d1d-325a410ffba8&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778750451_P3SWBWuKNu4SSpWs</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/68+COFFEE+%26+TEA/@16.0532582,108.2464907,17.82z/data=!4m6!3m5!1s0x314217001c0d52a5:0xb08551f1c1f5b871!8m2!3d16.053615!4d108.2466828!16s%2Fg%2F11yzrdtzh0?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">125HNH Homestay
+</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1556187895484884653?adults=5&amp;check_in=2026-07-29&amp;check_out=2026-08-01&amp;search_mode=regular_search&amp;source_impression_id=p3_1778741985_P38laXBpbm4dgmkg&amp;previous_page_section_name=1000&amp;federated_search_id=eae37c30-5b51-4642-bae5-466b5db5b0ec</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1556187895484884653/original/7cf07fb7-16fe-454f-bf6f-9476047cb688.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>Mewah, rumah 3 lt, di tengah2 da nang, deket bandara</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/16.060063,+108.186672?entry=tts&amp;g_ep=EgoyMDI2MDUxMS4wIPu8ASoASAFQAw%3D%3D&amp;skid=f77f9461-edca-4267-8eab-d2e5f3c7836d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gemini/Apt30m2/2ndBenThanhMarket/Q1
+</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1363871836847372705?unique_share_id=e67c40e0-eb66-453f-8597-da1edbf70fad&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778751354_P3xsfI38iBgI0JS4</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1363871836847372705/original/142cb0f6-b0b2-42e6-896a-83425bcac0ef.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>Deket Ben Thanh market alias pusat kota, studio lt 8</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Pyramids+Restaurant+Halal+-+Middle+Eastern+Halal+Cuisine+%26+Arabic+Coffee+-+Ben+Thanh+Market+-+Tourists+in+Saigon+%7C+District+1/@10.7702105,106.7000776,20.36z/data=!4m9!1m2!2m1!1sle+chong+kie+ho+chi+minh!3m5!1s0x31752fcbafcb3c2b:0x71ce6a0be10dfbe0!8m2!3d10.7703643!4d106.7004126!16s%2Fg%2F11xflyz0cc?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lina Home 8 - Can ho 2PN+ Vinhomes Grand Park Q9
+</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1300502516731992466?unique_share_id=dab2fb99-39d6-44ae-8303-065d37136db1&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778751900_P3_280VMiVHSXTOz</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-U3RheVN1cHBseUxpc3Rpbmc6MTMwMDUwMjUxNjczMTk5MjQ2Ng==/original/6d39fea5-f499-4f60-a67a-4ab73d74c70a.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Vinhomes+Grand+Park/@10.8363784,106.8398651,17z/data=!3m1!4b1!4m6!3m5!1s0x3175273121a14879:0x64cc5daec83c773!8m2!3d10.8363731!4d106.84244!16s%2Fg%2F11wvzvmg7t?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>Apartemen, terlihat bersih, vibes meikarta, 20 km ke Benh Thanh market</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 Cozy Studios for 5 pax near Ben Thanh &amp; Bui Vien
+</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/miso/Hosting-1430848393034237804/original/56fe0d70-8098-40f3-9d67-1f03035f196b.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1438029470295472414?unique_share_id=c7f7ce37-821e-4893-837d-2bce401bc060&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778752261_P3arOmiDDMWskPex</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/121%2F49+L%C3%AA+Th%E1%BB%8B+Ri%C3%AAng,+B%E1%BA%BFn+Th%C3%A0nh,+H%E1%BB%93+Ch%C3%AD+Minh,+Vietnam/@10.7700643,106.69074,20.23z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3d0126385d:0x269ab3b058ed3698!8m2!3d10.770318!4d106.6908484!16s%2Fg%2F11j8h0qfj2?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>Studio, 1.5 km dari Ben Thanh Market, perfect buat 3 guests???</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Downtown Duplex@BuiVien•4 Beds•Lift•Washer•Kitchen
+</t>
+  </si>
+  <si>
+    <t>Duplex, Vibes guyub dapet alias kasur mepet2, 5 menit ke Ben Thanh Market</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1590214868564972020?unique_share_id=ad8cd489-a93a-4b18-8aae-a160b556a3ad&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778752674_P3dSWUWuBViAwVIp</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1590214868564972020/original/d74dca73-93b4-4257-bcce-2f3cd538941d.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/C.Macro+Th%E1%BB%B1c+D%C6%B0%E1%BB%A1ng+S%E1%BA%A1ch+Vi%E1%BB%87t+Nam/@10.7639029,106.6927615,21z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752fb16bf8f9ad:0xa4de8d3544f2558a!8m2!3d10.7640143!4d106.692973!16s%2Fg%2F11g07s3lhd?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D1 Big Group Stay/8Pax/5Beds/2WC/Laundry/Kitchen
+</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1656462355120836879?unique_share_id=cfddc127-f55a-4079-a524-7095a81405c5&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778752688_P3W2Nce8zSWJKcor</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1656462355120836879/original/a84acb9e-3bb6-4cf5-b997-56a292b6aca2.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>Duplex, 7 menit ke Ben Thanh market, ada proyektor, unit baru</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/229+Pham+Ngu+Lao/@10.767733,106.6914827,18.95z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3df2e2bc1b:0xf5b67606e28b5f25!8m2!3d10.7682962!4d106.6926399!16s%2Fg%2F11z5nct8zk?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -411,7 +600,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -448,6 +637,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -691,7 +886,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
@@ -1554,6 +1749,654 @@
       <c r="Q17" s="13" t="s">
         <v>81</v>
       </c>
+    </row>
+    <row r="18" spans="1:17" ht="51">
+      <c r="A18" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" t="s">
+        <v>100</v>
+      </c>
+      <c r="C18" s="11">
+        <v>2</v>
+      </c>
+      <c r="D18" s="11">
+        <v>3</v>
+      </c>
+      <c r="E18" s="11">
+        <v>6</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J18" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K18" s="7">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="L18" s="7">
+        <v>35</v>
+      </c>
+      <c r="M18" s="15">
+        <v>825000</v>
+      </c>
+      <c r="N18" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="O18" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="P18" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q18" s="16" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="76.5">
+      <c r="A19" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>105</v>
+      </c>
+      <c r="C19" s="11">
+        <v>2</v>
+      </c>
+      <c r="D19" s="11">
+        <v>2</v>
+      </c>
+      <c r="E19" s="11">
+        <v>6</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K19" s="7">
+        <v>4.8</v>
+      </c>
+      <c r="L19" s="7">
+        <v>25</v>
+      </c>
+      <c r="M19" s="15">
+        <v>1122000</v>
+      </c>
+      <c r="N19" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="O19" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="P19" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q19" s="16" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="102">
+      <c r="A20" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="C20" s="11">
+        <v>2</v>
+      </c>
+      <c r="D20" s="11">
+        <v>1</v>
+      </c>
+      <c r="E20" s="11">
+        <v>6</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J20" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K20" s="7">
+        <v>4.88</v>
+      </c>
+      <c r="L20" s="7">
+        <v>34</v>
+      </c>
+      <c r="M20" s="15">
+        <v>984000</v>
+      </c>
+      <c r="N20" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="O20" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="P20" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q20" s="16" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="89.25">
+      <c r="A21" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="C21" s="11">
+        <v>2</v>
+      </c>
+      <c r="D21" s="11">
+        <v>2</v>
+      </c>
+      <c r="E21" s="11">
+        <v>5</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K21" s="7">
+        <v>4.8600000000000003</v>
+      </c>
+      <c r="L21" s="7">
+        <v>104</v>
+      </c>
+      <c r="M21" s="15">
+        <v>995000</v>
+      </c>
+      <c r="N21" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="O21" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="P21" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q21" s="16" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="51">
+      <c r="A22" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C22" s="11">
+        <v>3</v>
+      </c>
+      <c r="D22" s="11">
+        <v>3</v>
+      </c>
+      <c r="E22" s="11">
+        <v>7</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I22" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J22" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K22" s="7">
+        <v>4.6399999999999997</v>
+      </c>
+      <c r="L22" s="7">
+        <v>33</v>
+      </c>
+      <c r="M22" s="15">
+        <v>1023000</v>
+      </c>
+      <c r="N22" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="O22" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="P22" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q22" s="16" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="51">
+      <c r="A23" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="C23" s="11">
+        <v>2</v>
+      </c>
+      <c r="D23" s="11">
+        <v>1</v>
+      </c>
+      <c r="E23" s="11">
+        <v>5</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I23" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J23" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K23" s="7">
+        <v>5</v>
+      </c>
+      <c r="L23" s="7">
+        <v>3</v>
+      </c>
+      <c r="M23" s="15">
+        <v>800000</v>
+      </c>
+      <c r="N23" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="O23" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="P23" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q23" s="16" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="63.75">
+      <c r="A24" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="C24" s="11">
+        <v>3</v>
+      </c>
+      <c r="D24" s="11">
+        <v>3</v>
+      </c>
+      <c r="E24" s="11">
+        <v>7</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I24" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K24" s="7">
+        <v>5</v>
+      </c>
+      <c r="L24" s="7">
+        <v>9</v>
+      </c>
+      <c r="M24" s="15">
+        <v>1259000</v>
+      </c>
+      <c r="N24" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="O24" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="P24" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q24" s="16" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="63.75">
+      <c r="A25" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C25" s="11">
+        <v>3</v>
+      </c>
+      <c r="D25" s="11">
+        <v>1</v>
+      </c>
+      <c r="E25" s="11">
+        <v>5</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I25" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J25" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K25" s="7">
+        <v>4.83</v>
+      </c>
+      <c r="L25" s="7">
+        <v>58</v>
+      </c>
+      <c r="M25" s="15">
+        <v>842000</v>
+      </c>
+      <c r="N25" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="O25" s="16" t="s">
+        <v>136</v>
+      </c>
+      <c r="P25" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q25" s="16" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" ht="76.5">
+      <c r="A26" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="C26" s="11">
+        <v>3</v>
+      </c>
+      <c r="D26" s="11">
+        <v>2</v>
+      </c>
+      <c r="E26" s="11">
+        <v>6</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J26" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K26" s="7">
+        <v>5</v>
+      </c>
+      <c r="L26" s="7">
+        <v>30</v>
+      </c>
+      <c r="M26" s="15">
+        <v>708000</v>
+      </c>
+      <c r="N26" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="O26" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="P26" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q26" s="16" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="76.5">
+      <c r="A27" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="C27" s="11">
+        <v>2</v>
+      </c>
+      <c r="D27" s="11">
+        <v>2</v>
+      </c>
+      <c r="E27" s="11">
+        <v>5</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I27" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J27" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K27" s="7">
+        <v>5</v>
+      </c>
+      <c r="L27" s="7">
+        <v>3</v>
+      </c>
+      <c r="M27" s="15">
+        <v>923000</v>
+      </c>
+      <c r="N27" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="O27" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="P27" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q27" s="16" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="76.5">
+      <c r="A28" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="C28" s="11">
+        <v>4</v>
+      </c>
+      <c r="D28" s="11">
+        <v>1</v>
+      </c>
+      <c r="E28" s="11">
+        <v>8</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I28" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J28" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K28" s="7">
+        <v>4.7300000000000004</v>
+      </c>
+      <c r="L28" s="7">
+        <v>15</v>
+      </c>
+      <c r="M28" s="15">
+        <v>984000</v>
+      </c>
+      <c r="N28" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="O28" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="P28" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q28" s="16" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="76.5">
+      <c r="A29" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="C29" s="11">
+        <v>5</v>
+      </c>
+      <c r="D29" s="11">
+        <v>2</v>
+      </c>
+      <c r="E29" s="11">
+        <v>8</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H29" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I29" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J29" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K29" s="7">
+        <v>5</v>
+      </c>
+      <c r="L29" s="7">
+        <v>2</v>
+      </c>
+      <c r="M29" s="15">
+        <v>1190000</v>
+      </c>
+      <c r="N29" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="O29" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="P29" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q29" s="16" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17">
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+    </row>
+    <row r="31" spans="1:17">
+      <c r="H31" s="9"/>
+      <c r="I31" s="9"/>
+    </row>
+    <row r="32" spans="1:17">
+      <c r="H32" s="9"/>
+      <c r="I32" s="9"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1594,6 +2437,41 @@
     <hyperlink ref="Q17" r:id="rId35" xr:uid="{F4651035-85EE-4C69-A618-11337D5578FD}"/>
     <hyperlink ref="P4" r:id="rId36" xr:uid="{44258B57-2022-4512-8B2A-635A07EBD702}"/>
     <hyperlink ref="P3" r:id="rId37" display="https://google.com/maps/place/Mercury+Beach+House/@16.0884991,108.2460601,17z/data=!4m10!3m9!1s0x314217f213c3031f:0xc3fa594a2c3558c1!5m2!4m1!1i2!8m2!3d16.0884991!4d108.248635!15sCjRNZXJjdXJ5IEJlYWNoIHdpdGggMkJScy0zIEJlZHMtUE9PTCAxMG0gdG8gdGhlIGJlYWNokgEFaG90ZWzgAQA!16s%2Fg%2F11jsp4x6y6?entry=tts&amp;g_ep=EgoyMDI2MDUwMi4wIPu8ASoASAFQAw%3D%3D&amp;skid=1ede066e-c2ca-421e-b8be-8fb412b82088" xr:uid="{5E649388-17BD-4B9E-A309-83F73D732E56}"/>
+    <hyperlink ref="O18" r:id="rId38" xr:uid="{3091D75E-6088-4598-8E9F-AAED57F6C1BA}"/>
+    <hyperlink ref="Q18" r:id="rId39" xr:uid="{25F13F7C-12B6-437E-9A2B-B0DAF70F2289}"/>
+    <hyperlink ref="P18" r:id="rId40" xr:uid="{7C9ED5B5-E4F1-4017-B1AA-0ED1779D87A0}"/>
+    <hyperlink ref="O19" r:id="rId41" xr:uid="{02D47D6D-D06A-4E9B-89A3-1013A6528204}"/>
+    <hyperlink ref="Q19" r:id="rId42" xr:uid="{4058EB64-2805-4FB1-8891-6BE5ABA2BCF7}"/>
+    <hyperlink ref="O20" r:id="rId43" xr:uid="{E36242DA-FA92-435E-A4F4-5E09DBCC0459}"/>
+    <hyperlink ref="Q20" r:id="rId44" xr:uid="{1A85250B-E0EA-419A-8912-8E0070361A67}"/>
+    <hyperlink ref="P20" r:id="rId45" xr:uid="{BA88ECA5-3ED7-4453-9836-D0C2B7970406}"/>
+    <hyperlink ref="O21" r:id="rId46" xr:uid="{0DD9042B-7E82-4A1C-981B-95DC0F0E66E2}"/>
+    <hyperlink ref="Q21" r:id="rId47" xr:uid="{731BD421-991E-41A3-B362-526FFCECEF9A}"/>
+    <hyperlink ref="P21" r:id="rId48" xr:uid="{D7DB9A97-209E-4747-8DE8-F08B7B9C0EAD}"/>
+    <hyperlink ref="O22" r:id="rId49" xr:uid="{12642672-35BC-482A-9371-0E5DB74F5099}"/>
+    <hyperlink ref="Q22" r:id="rId50" xr:uid="{A5C81D10-C165-437B-901D-AA3EFB878EA0}"/>
+    <hyperlink ref="P22" r:id="rId51" display="https://www.google.com/maps/place/The+Wooden+Page/@16.0816664,108.2334076,19.91z/data=!4m17!1m7!3m6!1s0x3142192ea7af17a7:0xc89a2c1fa256fb94!2zUXXDoW4gTeG6uSBLZW4!8m2!3d16.0822394!4d108.2332973!16s%2Fg%2F11ststlgnz!3m8!1s0x31421793e1758355:0x8ed7d69dd01fc78b!5m2!4m1!1i2!8m2!3d16.081863!4d108.2338518!16s%2Fg%2F11tn6kcvmm?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{EA20416F-B46B-4593-9C4F-4619361E8A40}"/>
+    <hyperlink ref="Q23" r:id="rId52" xr:uid="{0D44DED3-15A4-4C70-ACF1-835EC9CB0784}"/>
+    <hyperlink ref="O23" r:id="rId53" xr:uid="{17523106-EB31-4F77-B3B9-4E991D3D0404}"/>
+    <hyperlink ref="P23" r:id="rId54" xr:uid="{2EFFCD1F-C2FA-41DA-935E-DD5036698130}"/>
+    <hyperlink ref="O24" r:id="rId55" display="https://www.airbnb.com/rooms/1556187895484884653?adults=5&amp;check_in=2026-07-29&amp;check_out=2026-08-01&amp;search_mode=regular_search&amp;source_impression_id=p3_1778741985_P38laXBpbm4dgmkg&amp;previous_page_section_name=1000&amp;federated_search_id=eae37c30-5b51-4642-bae5-466b5db5b0ec" xr:uid="{E1B7FA9C-616E-4E02-896F-089B47A5A934}"/>
+    <hyperlink ref="Q24" r:id="rId56" xr:uid="{1E0BF4EE-7FD2-413A-B8BC-17F888B9350C}"/>
+    <hyperlink ref="P24" r:id="rId57" xr:uid="{E0FB3868-609E-4B43-84BD-F2563B94E8FE}"/>
+    <hyperlink ref="O25" r:id="rId58" xr:uid="{9B5E18B5-8809-48EA-8F9C-9B2284647450}"/>
+    <hyperlink ref="Q25" r:id="rId59" xr:uid="{0C3F416E-D1C6-4038-900D-7FB07E51F560}"/>
+    <hyperlink ref="P25" r:id="rId60" display="https://www.google.com/maps/place/Pyramids+Restaurant+Halal+-+Middle+Eastern+Halal+Cuisine+%26+Arabic+Coffee+-+Ben+Thanh+Market+-+Tourists+in+Saigon+%7C+District+1/@10.7702105,106.7000776,20.36z/data=!4m9!1m2!2m1!1sle+chong+kie+ho+chi+minh!3m5!1s0x31752fcbafcb3c2b:0x71ce6a0be10dfbe0!8m2!3d10.7703643!4d106.7004126!16s%2Fg%2F11xflyz0cc?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{D022BFF9-C240-4D60-A3A0-B333C742D3C9}"/>
+    <hyperlink ref="O26" r:id="rId61" xr:uid="{29A8416D-BBCE-4236-BC58-637B32957D63}"/>
+    <hyperlink ref="Q26" r:id="rId62" xr:uid="{CD4A5948-5F18-4A06-86AC-0EF2FCEF752E}"/>
+    <hyperlink ref="P26" r:id="rId63" xr:uid="{75D88B4F-EB8E-4357-97C6-6EC93CCA55EB}"/>
+    <hyperlink ref="Q27" r:id="rId64" xr:uid="{D19B8FA7-95B8-4FF1-84CD-984128495F0A}"/>
+    <hyperlink ref="O27" r:id="rId65" xr:uid="{1E644DB5-138F-4514-87C1-8D01E021F60E}"/>
+    <hyperlink ref="P27" r:id="rId66" display="https://www.google.com/maps/place/121%2F49+L%C3%AA+Th%E1%BB%8B+Ri%C3%AAng,+B%E1%BA%BFn+Th%C3%A0nh,+H%E1%BB%93+Ch%C3%AD+Minh,+Vietnam/@10.7700643,106.69074,20.23z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3d0126385d:0x269ab3b058ed3698!8m2!3d10.770318!4d106.6908484!16s%2Fg%2F11j8h0qfj2?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{7834632D-5392-49B3-8759-ACE8294F0F5C}"/>
+    <hyperlink ref="O28" r:id="rId67" xr:uid="{B47D79C9-7FA4-4084-8A7F-3496B862703D}"/>
+    <hyperlink ref="Q28" r:id="rId68" xr:uid="{0556A8F5-98BB-4842-A77C-819650662487}"/>
+    <hyperlink ref="P28" r:id="rId69" display="https://www.google.com/maps/place/C.Macro+Th%E1%BB%B1c+D%C6%B0%E1%BB%A1ng+S%E1%BA%A1ch+Vi%E1%BB%87t+Nam/@10.7639029,106.6927615,21z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752fb16bf8f9ad:0xa4de8d3544f2558a!8m2!3d10.7640143!4d106.692973!16s%2Fg%2F11g07s3lhd?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{DA4CD0AD-171C-4E4A-ADB4-C8467F04EA19}"/>
+    <hyperlink ref="O29" r:id="rId70" xr:uid="{A201A6E0-4C43-489F-B008-F6087D50353A}"/>
+    <hyperlink ref="Q29" r:id="rId71" xr:uid="{4D02F78F-8922-4FAC-B501-69FD9E985CA3}"/>
+    <hyperlink ref="P29" r:id="rId72" display="https://www.google.com/maps/place/229+Pham+Ngu+Lao/@10.767733,106.6914827,18.95z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3df2e2bc1b:0xf5b67606e28b5f25!8m2!3d10.7682962!4d106.6926399!16s%2Fg%2F11z5nct8zk?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{D4453A9F-7434-43C4-91D7-143D85457C23}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Agoda and Trip columns to stays.xlsx
</commit_message>
<xml_diff>
--- a/stays.xlsx
+++ b/stays.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dika\belajar\Viet\stay_picker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E8DE25-939B-4751-B0A4-DE679F4711A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABDA40D5-FAE4-40F3-BEE1-3CE5FD0B84D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stays" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="206">
   <si>
     <t>FIXED: Sheet renamed to Stays. Distance categories corrected. Dana Home MT price fixed to 1600000. Yellow cells = corrected values.</t>
   </si>
@@ -510,13 +510,151 @@
   </si>
   <si>
     <t>https://www.google.com/maps/place/229+Pham+Ngu+Lao/@10.767733,106.6914827,18.95z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3df2e2bc1b:0xf5b67606e28b5f25!8m2!3d10.7682962!4d106.6926399!16s%2Fg%2F11z5nct8zk?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>The Quiet Elegance Apartment</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Lantai 32, Hostnya meyakinkan, di district 7</t>
+  </si>
+  <si>
+    <t>https://id.trip.com/hotels/Ho-Chi-Minh-City-hotel-detail-128244381/The-Quiet-Elegance-Apartment/?locale=en-ID&amp;fromfavorites=1&amp;tid=H0011_10650019167&amp;checkin=2026-08-01&amp;checkout=2026-08-03&amp;display=exavg&amp;crn=1&amp;adult=2&amp;children=0&amp;curr=IDR</t>
+  </si>
+  <si>
+    <t>Jessica's home in Soho Residence, District 1</t>
+  </si>
+  <si>
+    <t>Yes, Laundry room</t>
+  </si>
+  <si>
+    <t>Ada 6 properti gitu</t>
+  </si>
+  <si>
+    <t>https://id.trip.com/hotels/Ho-Chi-Minh-City-hotel-detail-105725759/Jessica%27s-home-in-Soho-Residence%2C-District-1/?locale=en-ID&amp;fromfavorites=1&amp;tid=H0011_10650019167&amp;checkin=2026-08-01&amp;checkout=2026-08-03&amp;display=exavg&amp;crn=1&amp;adult=2&amp;children=0&amp;curr=IDR</t>
+  </si>
+  <si>
+    <t>Yu Stay Soho Residence and Hotels</t>
+  </si>
+  <si>
+    <t>Yes, cleaning service</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>ada sofa bed, facilitynya kurang detil, ada di district 1</t>
+  </si>
+  <si>
+    <t>https://id.trip.com/hotels/Ho-Chi-Minh-City-hotel-detail-123688785/Yu-Stay-Soho-Residence-and-Hotels/?locale=en-ID&amp;fromfavorites=1&amp;tid=H0011_10650019167&amp;checkin=2026-08-01&amp;checkout=2026-08-03&amp;display=exavg&amp;crn=1&amp;adult=2&amp;children=0&amp;curr=IDR</t>
+  </si>
+  <si>
+    <t>Signy House Hotel &amp; Apartments - 15B Trần Khánh Dư</t>
+  </si>
+  <si>
+    <t>&gt;1 km</t>
+  </si>
+  <si>
+    <t>Ada family room (maks. 4 orang), masih perlu konfirmasi bisa extra bed atau tidak.</t>
+  </si>
+  <si>
+    <t>https://www.agoda.com/luxy-park-hotel-apartments-city-centre/hotel/ho-chi-minh-city-vn.html?locale=en-us&amp;ckuid=146075fe-8120-4edc-ba4d-4048de663867&amp;prid=0&amp;currency=IDR&amp;correlationId=03bbe63e-5401-44da-bf60-7fa802f25046&amp;analyticsSessionId=-6326601013581217769&amp;pageTypeId=7&amp;realLanguageId=1&amp;languageId=1&amp;origin=ID&amp;stateCode=JB&amp;cid=1918349&amp;userId=146075fe-8120-4edc-ba4d-4048de663867&amp;whitelabelid=1&amp;loginLvl=0&amp;storefrontId=3&amp;currencyId=25&amp;currencyCode=IDR&amp;htmlLanguage=en-us&amp;cultureInfoName=en-us&amp;machineName=sg-pc-6g-acm-web-user-7c49cd99bf-7q29g&amp;trafficGroupId=7&amp;trafficSubGroupId=200&amp;aid=102968&amp;useFullPageLogin=true&amp;cttp=4&amp;isRealUser=true&amp;mode=production&amp;browserFamily=Chrome&amp;cdnDomain=agoda.net&amp;checkIn=2026-08-01&amp;checkOut=2026-08-03&amp;rooms=2&amp;adults=5&amp;childs=0&amp;priceCur=IDR&amp;los=2&amp;textToSearch=Signy+House+Hotel+%26+Apartments&amp;productType=-1&amp;travellerType=3&amp;familyMode=off&amp;ds=nf5N%2FjXvFWrbhAxi</t>
+  </si>
+  <si>
+    <t>https://pix8.agoda.net/hotelImages/6915654/928817220/3423b19a83fde7b03d4f7cddac9e3b5e.jpg?ce=2&amp;s=1024x</t>
+  </si>
+  <si>
+    <t>42 Cocoon Danang Airport•Terminal Walk•City Center</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1667409155356761194?check_in=2026-07-30&amp;check_out=2026-08-01&amp;guests=1&amp;adults=5&amp;s=67&amp;unique_share_id=b12aabe2-aae9-47c4-8f31-ea24e9d38262</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1667409155356761194/original/d6f3feb0-4a7c-4ba5-a8c0-a3e6b3adc301.jpeg?im_w=1200</t>
+  </si>
+  <si>
+    <t>2BR 6G LUX Home in D3 | R2</t>
+  </si>
+  <si>
+    <t>Ye</t>
+  </si>
+  <si>
+    <t>Entire home, adanya di Distrik 3, ada UNO!!!</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1136142852152098662?check_in=2026-08-01&amp;check_out=2026-08-03&amp;guests=5&amp;adults=5&amp;s=67&amp;unique_share_id=78afa33c-6081-4a88-af73-56f495d8f4c9</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-U3RheVN1cHBseUxpc3Rpbmc6MTEzNjE0Mjg1MjE1MjA5ODY2Mg%3D%3D/original/67c792d2-0fe1-4da4-87e2-0aff5b5b108e.jpeg?im_w=1200</t>
+  </si>
+  <si>
+    <t>Stylish Loft 6Pax/3B/Laundry &amp; Dryer @BuiVien 300m</t>
+  </si>
+  <si>
+    <t>Tipe loft gitu (kamar atas bawah), duplex, ada airport pick up service, ada proyektor</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1414940410920129787?check_in=2026-08-01&amp;check_out=2026-08-03&amp;guests=5&amp;adults=5&amp;s=67&amp;unique_share_id=1e526ed1-0a9a-4042-814a-bce4dd9b97da</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1414940410920129787/original/2ecedd03-5d80-4844-bf71-c050c019d364.jpeg?im_w=1200</t>
+  </si>
+  <si>
+    <t>6pax - 3BR Apartment Centre D1</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Smoking di balkon, kamar di lantai LIMA tapi aksesnya cuman pakai tangga</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1436726038481941526?check_in=2026-08-01&amp;check_out=2026-08-03&amp;guests=5&amp;adults=5&amp;s=67&amp;unique_share_id=63e0f203-e6d3-4f05-ac94-9d1da158e251</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-U3RheVN1cHBseUxpc3Rpbmc6MTQzNjcyNjAzODQ4MTk0MTUyNg==/original/e4b921a6-93aa-4f40-aca3-59c070bdc94c.jpeg?im_w=1200</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Signy+House+Hotel+%26+Apartments+-+15B+Tr%E1%BA%A7n+Kh%C3%A1nh+D%C6%B0/@10.7937942,106.6782041,15z/data=!4m9!3m8!1s0x3175297257c4b02d:0xf2b70587ed8538c2!5m2!4m1!1i2!8m2!3d10.7937733!4d106.6884824!16s%2Fg%2F11fkgscnkj?entry=tts&amp;g_ep=EgoyMDI2MDUxMy4wIPu8ASoASAFQAw%3D%3D&amp;skid=47be7804-7c50-4e29-9594-7f7d7e9438b4</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/16%C2%B003'08.7%22N+108%C2%B012'14.5%22E/@16.052417,108.204016,17z/data=!3m1!4b1!4m4!3m3!8m2!3d16.052417!4d108.204016?entry=ttu&amp;g_ep=EgoyMDI2MDUxMy4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/10.786979,+106.677436?entry=tts&amp;g_ep=EgoyMDI2MDUxMy4wIPu8ASoASAFQAw%3D%3D&amp;skid=c2dafc2e-5783-4b29-abe2-5556b5978c67</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/202%2F5+C%C3%B4+B%E1%BA%AFc,+C%E1%BA%A7u+%C3%94ng+L%C3%A3nh,+H%E1%BB%93+Ch%C3%AD+Minh+70000,+Vietnam/@10.7636823,106.6930261,18.86z/data=!4m6!3m5!1s0x31752f169be87b2f:0xbcf056dae1984527!8m2!3d10.7639937!4d106.6935204!16s%2Fg%2F11x5gwft93?entry=tts&amp;g_ep=EgoyMDI2MDUxMy4wIPu8ASoASAFQAw%3D%3D&amp;skid=68804ac9-ef39-469c-9601-44cf2802946b</t>
+  </si>
+  <si>
+    <t>google.com/maps/place/18A%2F8%2F17+Nguyễn+Thị+Minh+Khai,+Sài+Gòn,+Hồ+Chí+Minh,+Vietnam/@10.7863952,106.6997079,19.77z/data=!4m6!3m5!1s0x31752f4a8072518f:0x68b294cadc3fdbae!8m2!3d10.7864684!4d106.6999852!16s%2Fg%2F11j2vtzy8y?entry=tts&amp;g_ep=EgoyMDI2MDUxMy4wIPu8ASoASAFQAw%3D%3D&amp;skid=22cb2197-8972-4286-a008-9909d8b2fa0e</t>
+  </si>
+  <si>
+    <t>https://aw-d.tripcdn.com/images/1mc1y12000kcqxxbeF15E_W_1280_853_R5.webp?proc=watermark/image_trip1,l_ne,x_16,y_16,w_67,h_16;digimark/t_image,logo_tripbinary;ignoredefaultwm,1A8F</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/C%C4%83n+H%E1%BB%99+Lavida+Plus+Qu%E1%BA%ADn+7/@10.7271647,106.6994728,16.77z/data=!4m6!3m5!1s0x31752ffb91d6c583:0xa398b70b12abf8dd!8m2!3d10.7272695!4d106.7018208!16s%2Fg%2F11m5y0434z?entry=ttu&amp;g_ep=EgoyMDI2MDUxMy4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>https://aw-d.tripcdn.com/images/1mc4z12000lg0a4geE21B_W_1280_853_R5.webp?proc=watermark/image_trip1,l_ne,x_16,y_16,w_67,h_16;digimark/t_image,logo_tripbinary;ignoredefaultwm,1A8F</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/H%E1%BB%93ng+Tr%C3%A0+Ng%C3%B4+Gia+H078/@10.7636066,106.6951405,20z/data=!4m6!3m5!1s0x31752fb67d1f4b5f:0x4cc87f858721ebe3!8m2!3d10.763715!4d106.69538!16s%2Fg%2F11t0rz2fvv?entry=ttu&amp;g_ep=EgoyMDI2MDUxMy4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>https://aw-d.tripcdn.com/images/1z60j12000fqwckem7936_W_1280_853_R5.webp?proc=watermark/image_trip1,l_ne,x_16,y_16,w_67,h_16;digimark/t_image,logo_tripbinary;ignoredefaultwm,1A8F</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/SOHO+Residence+%26+Hotel/@10.7635401,106.6944889,19.32z/data=!4m17!1m7!3m6!1s0x31752fb67d1f4b5f:0x4cc87f858721ebe3!2zSOG7k25nIFRyw6AgTmfDtCBHaWEgSDA3OA!8m2!3d10.763715!4d106.69538!16s%2Fg%2F11t0rz2fvv!3m8!1s0x31752f2748bdb637:0xd9b23c45d5aa6af4!5m2!4m1!1i2!8m2!3d10.7636913!4d106.6946027!16s%2Fg%2F11tmybkj_w?entry=ttu&amp;g_ep=EgoyMDI2MDUxMy4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -567,6 +705,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -600,7 +751,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -642,8 +793,35 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -886,8 +1064,8 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q32"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75"/>
+  <dimension ref="A1:Q37"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="29.7109375" customWidth="1"/>
@@ -897,12 +1075,12 @@
     <col min="17" max="17" width="31.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
@@ -955,7 +1133,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="153">
+    <row r="3" spans="1:17" ht="153" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -1008,7 +1186,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="127.5">
+    <row r="4" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
@@ -1061,7 +1239,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="114.75">
+    <row r="5" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -1114,7 +1292,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="140.25">
+    <row r="6" spans="1:17" ht="140.25" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -1167,7 +1345,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="114.75">
+    <row r="7" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -1220,7 +1398,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="114.75">
+    <row r="8" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
@@ -1273,7 +1451,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="127.5">
+    <row r="9" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
@@ -1326,7 +1504,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="127.5">
+    <row r="10" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -1379,7 +1557,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="114.75">
+    <row r="11" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>56</v>
       </c>
@@ -1432,7 +1610,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="114.75">
+    <row r="12" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>56</v>
       </c>
@@ -1485,7 +1663,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="114.75">
+    <row r="13" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>18</v>
       </c>
@@ -1538,7 +1716,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="114.75">
+    <row r="14" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>18</v>
       </c>
@@ -1591,7 +1769,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="114.75">
+    <row r="15" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>18</v>
       </c>
@@ -1644,7 +1822,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="76.5">
+    <row r="16" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
         <v>18</v>
       </c>
@@ -1697,7 +1875,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="127.5">
+    <row r="17" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>56</v>
       </c>
@@ -1750,7 +1928,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="51">
+    <row r="18" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
         <v>18</v>
       </c>
@@ -1803,7 +1981,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="19" spans="1:17" ht="76.5">
+    <row r="19" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
         <v>18</v>
       </c>
@@ -1856,11 +2034,11 @@
         <v>108</v>
       </c>
     </row>
-    <row r="20" spans="1:17" ht="102">
+    <row r="20" spans="1:17" ht="102" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="7" t="s">
         <v>110</v>
       </c>
       <c r="C20" s="11">
@@ -1909,7 +2087,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="21" spans="1:17" ht="89.25">
+    <row r="21" spans="1:17" ht="89.25" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>18</v>
       </c>
@@ -1962,7 +2140,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="51">
+    <row r="22" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>18</v>
       </c>
@@ -2015,7 +2193,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="23" spans="1:17" ht="51">
+    <row r="23" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>18</v>
       </c>
@@ -2068,7 +2246,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="24" spans="1:17" ht="63.75">
+    <row r="24" spans="1:17" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
         <v>18</v>
       </c>
@@ -2121,7 +2299,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="63.75">
+    <row r="25" spans="1:17" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>56</v>
       </c>
@@ -2174,7 +2352,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="76.5">
+    <row r="26" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
         <v>56</v>
       </c>
@@ -2227,7 +2405,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="27" spans="1:17" ht="76.5">
+    <row r="27" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
         <v>56</v>
       </c>
@@ -2280,7 +2458,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="76.5">
+    <row r="28" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
         <v>56</v>
       </c>
@@ -2333,7 +2511,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="29" spans="1:17" ht="76.5">
+    <row r="29" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
         <v>56</v>
       </c>
@@ -2386,17 +2564,429 @@
         <v>157</v>
       </c>
     </row>
-    <row r="30" spans="1:17">
-      <c r="H30" s="9"/>
-      <c r="I30" s="9"/>
-    </row>
-    <row r="31" spans="1:17">
-      <c r="H31" s="9"/>
-      <c r="I31" s="9"/>
-    </row>
-    <row r="32" spans="1:17">
-      <c r="H32" s="9"/>
-      <c r="I32" s="9"/>
+    <row r="30" spans="1:17" ht="51" x14ac:dyDescent="0.2">
+      <c r="A30" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="C30" s="21">
+        <v>3</v>
+      </c>
+      <c r="D30" s="21">
+        <v>3</v>
+      </c>
+      <c r="E30" s="21">
+        <v>6</v>
+      </c>
+      <c r="F30" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="G30" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="H30" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="I30" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="J30" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="K30" s="18">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="L30" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="M30" s="22">
+        <v>1018500</v>
+      </c>
+      <c r="N30" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="O30" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="P30" s="23" t="s">
+        <v>201</v>
+      </c>
+      <c r="Q30" s="23" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A31" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="C31" s="21">
+        <v>2</v>
+      </c>
+      <c r="D31" s="21">
+        <v>2</v>
+      </c>
+      <c r="E31" s="21">
+        <v>5</v>
+      </c>
+      <c r="F31" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="G31" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="H31" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="I31" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="J31" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="K31" s="18">
+        <v>4.55</v>
+      </c>
+      <c r="L31" s="20">
+        <v>153</v>
+      </c>
+      <c r="M31" s="22">
+        <v>1144500</v>
+      </c>
+      <c r="N31" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="O31" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="P31" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="Q31" s="23" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A32" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="C32" s="21">
+        <v>2</v>
+      </c>
+      <c r="D32" s="21">
+        <v>2</v>
+      </c>
+      <c r="E32" s="21">
+        <v>5</v>
+      </c>
+      <c r="F32" s="20" t="s">
+        <v>169</v>
+      </c>
+      <c r="G32" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="H32" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="I32" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="J32" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="K32" s="18">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="L32" s="20">
+        <v>53</v>
+      </c>
+      <c r="M32" s="22">
+        <v>1081000</v>
+      </c>
+      <c r="N32" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="O32" s="23" t="s">
+        <v>172</v>
+      </c>
+      <c r="P32" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q32" s="23" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" ht="331.5" x14ac:dyDescent="0.2">
+      <c r="A33" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="B33" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="C33" s="26">
+        <v>2</v>
+      </c>
+      <c r="D33" s="26">
+        <v>2</v>
+      </c>
+      <c r="E33" s="26">
+        <v>4</v>
+      </c>
+      <c r="F33" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="G33" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="H33" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I33" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="J33" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="K33" s="26">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="L33" s="26">
+        <v>94</v>
+      </c>
+      <c r="M33" s="28">
+        <v>780173</v>
+      </c>
+      <c r="N33" s="24" t="s">
+        <v>175</v>
+      </c>
+      <c r="O33" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="P33" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q33" s="27" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" ht="89.25" x14ac:dyDescent="0.2">
+      <c r="A34" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34" s="24" t="s">
+        <v>178</v>
+      </c>
+      <c r="C34" s="26">
+        <v>2</v>
+      </c>
+      <c r="D34" s="26">
+        <v>2</v>
+      </c>
+      <c r="E34" s="26">
+        <v>5</v>
+      </c>
+      <c r="F34" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="G34" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="H34" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I34" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="J34" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="K34" s="26">
+        <v>5</v>
+      </c>
+      <c r="L34" s="26">
+        <v>7</v>
+      </c>
+      <c r="M34" s="28">
+        <v>770578</v>
+      </c>
+      <c r="N34" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="O34" s="27" t="s">
+        <v>179</v>
+      </c>
+      <c r="P34" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="Q34" s="27" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A35" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="24" t="s">
+        <v>181</v>
+      </c>
+      <c r="C35" s="26">
+        <v>2</v>
+      </c>
+      <c r="D35" s="26">
+        <v>3</v>
+      </c>
+      <c r="E35" s="26">
+        <v>6</v>
+      </c>
+      <c r="F35" s="26" t="s">
+        <v>182</v>
+      </c>
+      <c r="G35" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="H35" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I35" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="J35" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="K35" s="26">
+        <v>4.95</v>
+      </c>
+      <c r="L35" s="26">
+        <v>37</v>
+      </c>
+      <c r="M35" s="28">
+        <v>949016.5</v>
+      </c>
+      <c r="N35" s="24" t="s">
+        <v>183</v>
+      </c>
+      <c r="O35" s="27" t="s">
+        <v>184</v>
+      </c>
+      <c r="P35" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q35" s="27" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
+      <c r="A36" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="B36" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="C36" s="26">
+        <v>1</v>
+      </c>
+      <c r="D36" s="26">
+        <v>3</v>
+      </c>
+      <c r="E36" s="26">
+        <v>6</v>
+      </c>
+      <c r="F36" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="H36" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I36" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="J36" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="K36" s="26">
+        <v>4.7699999999999996</v>
+      </c>
+      <c r="L36" s="26">
+        <v>30</v>
+      </c>
+      <c r="M36" s="28">
+        <v>986064.5</v>
+      </c>
+      <c r="N36" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="O36" s="27" t="s">
+        <v>188</v>
+      </c>
+      <c r="P36" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q36" s="27" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" ht="102" x14ac:dyDescent="0.2">
+      <c r="A37" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="B37" s="24" t="s">
+        <v>190</v>
+      </c>
+      <c r="C37" s="26">
+        <v>3</v>
+      </c>
+      <c r="D37" s="26">
+        <v>3</v>
+      </c>
+      <c r="E37" s="26">
+        <v>6</v>
+      </c>
+      <c r="F37" s="26" t="s">
+        <v>191</v>
+      </c>
+      <c r="G37" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="H37" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I37" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="J37" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="K37" s="26">
+        <v>4.58</v>
+      </c>
+      <c r="L37" s="26">
+        <v>33</v>
+      </c>
+      <c r="M37" s="28">
+        <v>972238</v>
+      </c>
+      <c r="N37" s="24" t="s">
+        <v>192</v>
+      </c>
+      <c r="O37" s="27" t="s">
+        <v>193</v>
+      </c>
+      <c r="P37" s="27" t="s">
+        <v>199</v>
+      </c>
+      <c r="Q37" s="27" t="s">
+        <v>194</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2472,6 +3062,28 @@
     <hyperlink ref="O29" r:id="rId70" xr:uid="{A201A6E0-4C43-489F-B008-F6087D50353A}"/>
     <hyperlink ref="Q29" r:id="rId71" xr:uid="{4D02F78F-8922-4FAC-B501-69FD9E985CA3}"/>
     <hyperlink ref="P29" r:id="rId72" display="https://www.google.com/maps/place/229+Pham+Ngu+Lao/@10.767733,106.6914827,18.95z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3df2e2bc1b:0xf5b67606e28b5f25!8m2!3d10.7682962!4d106.6926399!16s%2Fg%2F11z5nct8zk?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{D4453A9F-7434-43C4-91D7-143D85457C23}"/>
+    <hyperlink ref="P33" r:id="rId73" display="https://www.google.com/maps/place/Signy+House+Hotel+%26+Apartments+-+15B+Tr%E1%BA%A7n+Kh%C3%A1nh+D%C6%B0/@10.7937942,106.6782041,15z/data=!4m9!3m8!1s0x3175297257c4b02d:0xf2b70587ed8538c2!5m2!4m1!1i2!8m2!3d10.7937733!4d106.6884824!16s%2Fg%2F11fkgscnkj?entry=tts&amp;g_ep=EgoyMDI2MDUxMy4wIPu8ASoASAFQAw%3D%3D&amp;skid=47be7804-7c50-4e29-9594-7f7d7e9438b4" xr:uid="{D5F0658E-83F9-4842-8E1B-C884A47FB73D}"/>
+    <hyperlink ref="Q33" r:id="rId74" xr:uid="{1A8C3643-1642-451E-9410-6CF9FFEC2D94}"/>
+    <hyperlink ref="Q34" r:id="rId75" xr:uid="{C53609F4-15E7-4443-B02F-0C74133BB825}"/>
+    <hyperlink ref="O34" r:id="rId76" xr:uid="{3AC6E81A-6881-4337-8506-B3D382C7CF17}"/>
+    <hyperlink ref="P34" r:id="rId77" xr:uid="{687A6D4C-311E-495B-B859-7DC574CC4A73}"/>
+    <hyperlink ref="O35" r:id="rId78" xr:uid="{1FA4B93F-03BC-48A9-8B51-50064FF7FE02}"/>
+    <hyperlink ref="Q35" r:id="rId79" xr:uid="{A5F8DC54-E881-4FCB-9159-36AD18BF83BA}"/>
+    <hyperlink ref="P35" r:id="rId80" xr:uid="{A32DF229-EDA9-4BC6-ADE4-599B1CA01F6B}"/>
+    <hyperlink ref="O36" r:id="rId81" xr:uid="{E550138A-19A3-4433-933A-9E1E3665AFD8}"/>
+    <hyperlink ref="Q36" r:id="rId82" xr:uid="{DE0FF8BC-6382-4390-8FFB-A33701AE1678}"/>
+    <hyperlink ref="P36" r:id="rId83" display="https://maps.app.goo.gl/BoXEQmtD7p7UBWQF9" xr:uid="{3E71EB02-0A48-463C-BD49-37B122A1E55C}"/>
+    <hyperlink ref="O37" r:id="rId84" xr:uid="{83E719A9-EBF2-4255-8E50-F1AFDD3DEB65}"/>
+    <hyperlink ref="Q37" r:id="rId85" xr:uid="{049758F8-0E93-4846-AF70-5FFC65C94ABA}"/>
+    <hyperlink ref="P37" r:id="rId86" display="https://maps.app.goo.gl/8CGQz8X495XTkWsG6" xr:uid="{7628EC14-1A53-4FF5-94FD-C8B5E44766D9}"/>
+    <hyperlink ref="O30" r:id="rId87" xr:uid="{50B44A8F-1E12-43F2-8CE1-88FBDBCB2862}"/>
+    <hyperlink ref="O31" r:id="rId88" xr:uid="{E6A06F26-4042-4F78-98CB-A4703A09D563}"/>
+    <hyperlink ref="O32" r:id="rId89" xr:uid="{BB03F22A-3802-4705-A436-312DA30713C2}"/>
+    <hyperlink ref="Q30" r:id="rId90" xr:uid="{BE32A7B1-BB98-49B1-B4DF-3E2676C5EAAD}"/>
+    <hyperlink ref="P30" r:id="rId91" display="https://www.google.com/maps/place/C%C4%83n+H%E1%BB%99+Lavida+Plus+Qu%E1%BA%ADn+7/@10.7271647,106.6994728,16.77z/data=!4m6!3m5!1s0x31752ffb91d6c583:0xa398b70b12abf8dd!8m2!3d10.7272695!4d106.7018208!16s%2Fg%2F11m5y0434z?entry=ttu&amp;g_ep=EgoyMDI2MDUxMy4wIKXMDSoASAFQAw%3D%3D" xr:uid="{C367F6F5-5149-41FF-934E-A36B4A5B4344}"/>
+    <hyperlink ref="Q31" r:id="rId92" xr:uid="{F0DAF66C-579C-42A1-B3A3-563254C38222}"/>
+    <hyperlink ref="P31" r:id="rId93" display="https://www.google.com/maps/place/H%E1%BB%93ng+Tr%C3%A0+Ng%C3%B4+Gia+H078/@10.7636066,106.6951405,20z/data=!4m6!3m5!1s0x31752fb67d1f4b5f:0x4cc87f858721ebe3!8m2!3d10.763715!4d106.69538!16s%2Fg%2F11t0rz2fvv?entry=ttu&amp;g_ep=EgoyMDI2MDUxMy4wIKXMDSoASAFQAw%3D%3D" xr:uid="{4F1ED331-255E-45A6-B8C3-572C0191A949}"/>
+    <hyperlink ref="Q32" r:id="rId94" xr:uid="{50750A5D-2EAE-413E-9D75-3C11EC2D65F6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update stays.xlsx with Agoda and Trip columns
</commit_message>
<xml_diff>
--- a/stays.xlsx
+++ b/stays.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dika\belajar\Viet\stay_picker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABDA40D5-FAE4-40F3-BEE1-3CE5FD0B84D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF92E474-6370-4D42-8BAE-9B3060DA5F7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6615" yWindow="1860" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stays" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="208">
   <si>
     <t>FIXED: Sheet renamed to Stays. Distance categories corrected. Dana Home MT price fixed to 1600000. Yellow cells = corrected values.</t>
   </si>
@@ -648,6 +648,12 @@
   </si>
   <si>
     <t>https://www.google.com/maps/place/SOHO+Residence+%26+Hotel/@10.7635401,106.6944889,19.32z/data=!4m17!1m7!3m6!1s0x31752fb67d1f4b5f:0x4cc87f858721ebe3!2zSOG7k25nIFRyw6AgTmfDtCBHaWEgSDA3OA!8m2!3d10.763715!4d106.69538!16s%2Fg%2F11t0rz2fvv!3m8!1s0x31752f2748bdb637:0xd9b23c45d5aa6af4!5m2!4m1!1i2!8m2!3d10.7636913!4d106.6946027!16s%2Fg%2F11tmybkj_w?entry=ttu&amp;g_ep=EgoyMDI2MDUxMy4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>Agoda</t>
+  </si>
+  <si>
+    <t>Trip</t>
   </si>
 </sst>
 </file>
@@ -751,7 +757,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -796,18 +802,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1064,7 +1058,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q37"/>
+  <dimension ref="A1:S37"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
@@ -1073,14 +1067,16 @@
     <col min="15" max="15" width="34.42578125" customWidth="1"/>
     <col min="16" max="16" width="36.42578125" customWidth="1"/>
     <col min="17" max="17" width="31.28515625" customWidth="1"/>
+    <col min="18" max="18" width="31.140625" customWidth="1"/>
+    <col min="19" max="19" width="42.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
@@ -1127,13 +1123,19 @@
         <v>15</v>
       </c>
       <c r="P2" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="Q2" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="R2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="S2" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="153" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -1179,14 +1181,14 @@
       <c r="O3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="P3" s="13" t="s">
+      <c r="R3" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="Q3" s="1" t="s">
+      <c r="S3" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" ht="204" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
@@ -1232,14 +1234,14 @@
       <c r="O4" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P4" s="13" t="s">
+      <c r="R4" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="S4" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" ht="191.25" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -1285,14 +1287,14 @@
       <c r="O5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="P5" s="1" t="s">
+      <c r="R5" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="Q5" s="1" t="s">
+      <c r="S5" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="140.25" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" ht="344.25" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -1338,14 +1340,14 @@
       <c r="O6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="P6" s="1" t="s">
+      <c r="R6" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="Q6" s="1" t="s">
+      <c r="S6" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:19" ht="204" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -1391,14 +1393,14 @@
       <c r="O7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="P7" s="1" t="s">
+      <c r="R7" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="Q7" s="1" t="s">
+      <c r="S7" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:19" ht="344.25" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
@@ -1444,14 +1446,14 @@
       <c r="O8" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="P8" s="1" t="s">
+      <c r="R8" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="Q8" s="1" t="s">
+      <c r="S8" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:19" ht="306" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
@@ -1497,14 +1499,14 @@
       <c r="O9" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="P9" s="1" t="s">
+      <c r="R9" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="Q9" s="1" t="s">
+      <c r="S9" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:19" ht="395.25" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -1550,14 +1552,14 @@
       <c r="O10" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="P10" s="1" t="s">
+      <c r="R10" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="Q10" s="1" t="s">
+      <c r="S10" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:19" ht="191.25" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>56</v>
       </c>
@@ -1603,14 +1605,14 @@
       <c r="O11" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="P11" s="1" t="s">
+      <c r="R11" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="Q11" s="1" t="s">
+      <c r="S11" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:19" ht="178.5" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>56</v>
       </c>
@@ -1656,14 +1658,14 @@
       <c r="O12" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="P12" s="1" t="s">
+      <c r="R12" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="Q12" s="1" t="s">
+      <c r="S12" s="1" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:19" ht="369.75" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>18</v>
       </c>
@@ -1709,14 +1711,14 @@
       <c r="O13" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="P13" s="13" t="s">
+      <c r="R13" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="Q13" s="13" t="s">
+      <c r="S13" s="13" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:19" ht="178.5" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>18</v>
       </c>
@@ -1762,14 +1764,14 @@
       <c r="O14" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="P14" s="13" t="s">
+      <c r="R14" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="Q14" s="13" t="s">
+      <c r="S14" s="13" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="114.75" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:19" ht="178.5" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>18</v>
       </c>
@@ -1815,14 +1817,14 @@
       <c r="O15" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="P15" s="13" t="s">
+      <c r="R15" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="Q15" s="13" t="s">
+      <c r="S15" s="13" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:19" ht="178.5" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
         <v>18</v>
       </c>
@@ -1868,14 +1870,14 @@
       <c r="O16" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="P16" s="13" t="s">
+      <c r="R16" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="Q16" s="13" t="s">
+      <c r="S16" s="13" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:19" ht="357" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>56</v>
       </c>
@@ -1921,14 +1923,14 @@
       <c r="O17" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="P17" s="13" t="s">
+      <c r="R17" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="Q17" s="13" t="s">
+      <c r="S17" s="13" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="51" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
         <v>18</v>
       </c>
@@ -1974,14 +1976,14 @@
       <c r="O18" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="P18" s="16" t="s">
+      <c r="R18" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="Q18" s="16" t="s">
+      <c r="S18" s="16" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="19" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:19" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
         <v>18</v>
       </c>
@@ -2027,14 +2029,14 @@
       <c r="O19" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="P19" s="14" t="s">
+      <c r="R19" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="Q19" s="16" t="s">
+      <c r="S19" s="16" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="20" spans="1:17" ht="102" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
         <v>18</v>
       </c>
@@ -2080,14 +2082,14 @@
       <c r="O20" s="16" t="s">
         <v>111</v>
       </c>
-      <c r="P20" s="16" t="s">
+      <c r="R20" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="Q20" s="16" t="s">
+      <c r="S20" s="16" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="21" spans="1:17" ht="89.25" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:19" ht="89.25" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>18</v>
       </c>
@@ -2133,14 +2135,14 @@
       <c r="O21" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="P21" s="16" t="s">
+      <c r="R21" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="Q21" s="16" t="s">
+      <c r="S21" s="16" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="51" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>18</v>
       </c>
@@ -2186,14 +2188,14 @@
       <c r="O22" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="P22" s="16" t="s">
+      <c r="R22" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="Q22" s="16" t="s">
+      <c r="S22" s="16" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="23" spans="1:17" ht="51" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>18</v>
       </c>
@@ -2239,14 +2241,14 @@
       <c r="O23" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="P23" s="16" t="s">
+      <c r="R23" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="Q23" s="16" t="s">
+      <c r="S23" s="16" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="24" spans="1:17" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:19" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
         <v>18</v>
       </c>
@@ -2292,14 +2294,14 @@
       <c r="O24" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="P24" s="16" t="s">
+      <c r="R24" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="Q24" s="16" t="s">
+      <c r="S24" s="16" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:19" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>56</v>
       </c>
@@ -2345,14 +2347,14 @@
       <c r="O25" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="P25" s="16" t="s">
+      <c r="R25" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="Q25" s="16" t="s">
+      <c r="S25" s="16" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:19" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
         <v>56</v>
       </c>
@@ -2398,14 +2400,14 @@
       <c r="O26" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="P26" s="16" t="s">
+      <c r="R26" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="Q26" s="16" t="s">
+      <c r="S26" s="16" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="27" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:19" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
         <v>56</v>
       </c>
@@ -2451,14 +2453,14 @@
       <c r="O27" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="P27" s="16" t="s">
+      <c r="R27" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="Q27" s="16" t="s">
+      <c r="S27" s="16" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:19" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
         <v>56</v>
       </c>
@@ -2504,14 +2506,14 @@
       <c r="O28" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="P28" s="16" t="s">
+      <c r="R28" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="Q28" s="16" t="s">
+      <c r="S28" s="16" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="29" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:19" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
         <v>56</v>
       </c>
@@ -2557,533 +2559,533 @@
       <c r="O29" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="P29" s="16" t="s">
+      <c r="R29" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="Q29" s="16" t="s">
+      <c r="S29" s="16" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="30" spans="1:17" ht="51" x14ac:dyDescent="0.2">
-      <c r="A30" s="21" t="s">
+    <row r="30" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+      <c r="A30" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B30" s="19" t="s">
+      <c r="B30" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="C30" s="21">
+      <c r="C30" s="11">
         <v>3</v>
       </c>
-      <c r="D30" s="21">
+      <c r="D30" s="11">
         <v>3</v>
       </c>
-      <c r="E30" s="21">
+      <c r="E30" s="11">
         <v>6</v>
       </c>
-      <c r="F30" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="G30" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="H30" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="I30" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="J30" s="20" t="s">
+      <c r="F30" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="I30" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J30" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="K30" s="18">
+      <c r="K30">
         <v>4.9000000000000004</v>
       </c>
-      <c r="L30" s="20" t="s">
+      <c r="L30" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="M30" s="22">
+      <c r="M30" s="15">
         <v>1018500</v>
       </c>
-      <c r="N30" s="20" t="s">
+      <c r="N30" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="O30" s="23" t="s">
+      <c r="Q30" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="P30" s="23" t="s">
+      <c r="R30" s="16" t="s">
         <v>201</v>
       </c>
-      <c r="Q30" s="23" t="s">
+      <c r="S30" s="16" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A31" s="21" t="s">
+    <row r="31" spans="1:19" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A31" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="C31" s="21">
-        <v>2</v>
-      </c>
-      <c r="D31" s="21">
-        <v>2</v>
-      </c>
-      <c r="E31" s="21">
+      <c r="C31" s="11">
+        <v>2</v>
+      </c>
+      <c r="D31" s="11">
+        <v>2</v>
+      </c>
+      <c r="E31" s="11">
         <v>5</v>
       </c>
-      <c r="F31" s="20" t="s">
+      <c r="F31" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="G31" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="H31" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="I31" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="J31" s="20" t="s">
+      <c r="G31" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I31" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J31" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="K31" s="18">
+      <c r="K31">
         <v>4.55</v>
       </c>
-      <c r="L31" s="20">
+      <c r="L31" s="9">
         <v>153</v>
       </c>
-      <c r="M31" s="22">
+      <c r="M31" s="15">
         <v>1144500</v>
       </c>
-      <c r="N31" s="20" t="s">
+      <c r="N31" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="O31" s="23" t="s">
+      <c r="Q31" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="P31" s="23" t="s">
+      <c r="R31" s="16" t="s">
         <v>203</v>
       </c>
-      <c r="Q31" s="23" t="s">
+      <c r="S31" s="16" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="32" spans="1:17" ht="63.75" x14ac:dyDescent="0.2">
-      <c r="A32" s="21" t="s">
+    <row r="32" spans="1:19" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A32" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B32" s="18" t="s">
+      <c r="B32" t="s">
         <v>168</v>
       </c>
-      <c r="C32" s="21">
-        <v>2</v>
-      </c>
-      <c r="D32" s="21">
-        <v>2</v>
-      </c>
-      <c r="E32" s="21">
+      <c r="C32" s="11">
+        <v>2</v>
+      </c>
+      <c r="D32" s="11">
+        <v>2</v>
+      </c>
+      <c r="E32" s="11">
         <v>5</v>
       </c>
-      <c r="F32" s="20" t="s">
+      <c r="F32" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="G32" s="20" t="s">
+      <c r="G32" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="H32" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="I32" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="J32" s="20" t="s">
+      <c r="H32" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I32" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J32" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="K32" s="18">
+      <c r="K32">
         <v>4.5999999999999996</v>
       </c>
-      <c r="L32" s="20">
+      <c r="L32" s="9">
         <v>53</v>
       </c>
-      <c r="M32" s="22">
+      <c r="M32" s="15">
         <v>1081000</v>
       </c>
-      <c r="N32" s="20" t="s">
+      <c r="N32" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="O32" s="23" t="s">
+      <c r="Q32" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="P32" t="s">
+      <c r="R32" t="s">
         <v>205</v>
       </c>
-      <c r="Q32" s="23" t="s">
+      <c r="S32" s="16" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="33" spans="1:17" ht="331.5" x14ac:dyDescent="0.2">
-      <c r="A33" s="26" t="s">
+    <row r="33" spans="1:19" ht="306" x14ac:dyDescent="0.2">
+      <c r="A33" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="B33" s="24" t="s">
+      <c r="B33" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="C33" s="26">
-        <v>2</v>
-      </c>
-      <c r="D33" s="26">
-        <v>2</v>
-      </c>
-      <c r="E33" s="26">
+      <c r="C33" s="20">
+        <v>2</v>
+      </c>
+      <c r="D33" s="20">
+        <v>2</v>
+      </c>
+      <c r="E33" s="20">
         <v>4</v>
       </c>
-      <c r="F33" s="26" t="s">
-        <v>27</v>
-      </c>
-      <c r="G33" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="H33" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="I33" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="J33" s="26" t="s">
+      <c r="F33" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="G33" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="H33" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="I33" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="J33" s="20" t="s">
         <v>174</v>
       </c>
-      <c r="K33" s="26">
+      <c r="K33" s="20">
         <v>4.4000000000000004</v>
       </c>
-      <c r="L33" s="26">
+      <c r="L33" s="20">
         <v>94</v>
       </c>
-      <c r="M33" s="28">
+      <c r="M33" s="22">
         <v>780173</v>
       </c>
-      <c r="N33" s="24" t="s">
+      <c r="N33" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="O33" s="24" t="s">
+      <c r="P33" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="P33" s="17" t="s">
+      <c r="R33" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="Q33" s="27" t="s">
+      <c r="S33" s="21" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="34" spans="1:17" ht="89.25" x14ac:dyDescent="0.2">
-      <c r="A34" s="26" t="s">
+    <row r="34" spans="1:19" ht="242.25" x14ac:dyDescent="0.2">
+      <c r="A34" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B34" s="24" t="s">
+      <c r="B34" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="C34" s="26">
-        <v>2</v>
-      </c>
-      <c r="D34" s="26">
-        <v>2</v>
-      </c>
-      <c r="E34" s="26">
+      <c r="C34" s="20">
+        <v>2</v>
+      </c>
+      <c r="D34" s="20">
+        <v>2</v>
+      </c>
+      <c r="E34" s="20">
         <v>5</v>
       </c>
-      <c r="F34" s="26" t="s">
-        <v>27</v>
-      </c>
-      <c r="G34" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="H34" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="I34" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="J34" s="26" t="s">
+      <c r="F34" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="G34" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="H34" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="I34" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="J34" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="K34" s="26">
+      <c r="K34" s="20">
         <v>5</v>
       </c>
-      <c r="L34" s="26">
+      <c r="L34" s="20">
         <v>7</v>
       </c>
-      <c r="M34" s="28">
+      <c r="M34" s="22">
         <v>770578</v>
       </c>
-      <c r="N34" s="24" t="s">
+      <c r="N34" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="O34" s="27" t="s">
+      <c r="O34" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="P34" s="17" t="s">
+      <c r="R34" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="Q34" s="27" t="s">
+      <c r="S34" s="21" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="35" spans="1:17" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A35" s="26" t="s">
+    <row r="35" spans="1:19" ht="191.25" x14ac:dyDescent="0.2">
+      <c r="A35" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="B35" s="24" t="s">
+      <c r="B35" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="C35" s="26">
-        <v>2</v>
-      </c>
-      <c r="D35" s="26">
+      <c r="C35" s="20">
+        <v>2</v>
+      </c>
+      <c r="D35" s="20">
         <v>3</v>
       </c>
-      <c r="E35" s="26">
+      <c r="E35" s="20">
         <v>6</v>
       </c>
-      <c r="F35" s="26" t="s">
+      <c r="F35" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="G35" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="H35" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="I35" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="J35" s="26" t="s">
+      <c r="G35" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="H35" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="I35" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="J35" s="20" t="s">
         <v>174</v>
       </c>
-      <c r="K35" s="26">
+      <c r="K35" s="20">
         <v>4.95</v>
       </c>
-      <c r="L35" s="26">
+      <c r="L35" s="20">
         <v>37</v>
       </c>
-      <c r="M35" s="28">
+      <c r="M35" s="22">
         <v>949016.5</v>
       </c>
-      <c r="N35" s="24" t="s">
+      <c r="N35" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="O35" s="27" t="s">
+      <c r="O35" s="21" t="s">
         <v>184</v>
       </c>
-      <c r="P35" s="17" t="s">
+      <c r="R35" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="Q35" s="27" t="s">
+      <c r="S35" s="21" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
-      <c r="A36" s="26" t="s">
+    <row r="36" spans="1:19" ht="369.75" x14ac:dyDescent="0.2">
+      <c r="A36" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="24" t="s">
+      <c r="B36" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="C36" s="26">
+      <c r="C36" s="20">
         <v>1</v>
       </c>
-      <c r="D36" s="26">
+      <c r="D36" s="20">
         <v>3</v>
       </c>
-      <c r="E36" s="26">
+      <c r="E36" s="20">
         <v>6</v>
       </c>
-      <c r="F36" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="G36" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="H36" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="I36" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="J36" s="26" t="s">
+      <c r="F36" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="H36" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="I36" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="J36" s="20" t="s">
         <v>174</v>
       </c>
-      <c r="K36" s="26">
+      <c r="K36" s="20">
         <v>4.7699999999999996</v>
       </c>
-      <c r="L36" s="26">
+      <c r="L36" s="20">
         <v>30</v>
       </c>
-      <c r="M36" s="28">
+      <c r="M36" s="22">
         <v>986064.5</v>
       </c>
-      <c r="N36" s="24" t="s">
+      <c r="N36" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="O36" s="27" t="s">
+      <c r="O36" s="21" t="s">
         <v>188</v>
       </c>
-      <c r="P36" s="27" t="s">
+      <c r="R36" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="Q36" s="27" t="s">
+      <c r="S36" s="21" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="37" spans="1:17" ht="102" x14ac:dyDescent="0.2">
-      <c r="A37" s="26" t="s">
+    <row r="37" spans="1:19" ht="306" x14ac:dyDescent="0.2">
+      <c r="A37" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="B37" s="24" t="s">
+      <c r="B37" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="C37" s="26">
+      <c r="C37" s="20">
         <v>3</v>
       </c>
-      <c r="D37" s="26">
+      <c r="D37" s="20">
         <v>3</v>
       </c>
-      <c r="E37" s="26">
+      <c r="E37" s="20">
         <v>6</v>
       </c>
-      <c r="F37" s="26" t="s">
+      <c r="F37" s="20" t="s">
         <v>191</v>
       </c>
-      <c r="G37" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="H37" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="I37" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="J37" s="26" t="s">
+      <c r="G37" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="H37" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="I37" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="J37" s="20" t="s">
         <v>174</v>
       </c>
-      <c r="K37" s="26">
+      <c r="K37" s="20">
         <v>4.58</v>
       </c>
-      <c r="L37" s="26">
+      <c r="L37" s="20">
         <v>33</v>
       </c>
-      <c r="M37" s="28">
+      <c r="M37" s="22">
         <v>972238</v>
       </c>
-      <c r="N37" s="24" t="s">
+      <c r="N37" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="O37" s="27" t="s">
+      <c r="O37" s="21" t="s">
         <v>193</v>
       </c>
-      <c r="P37" s="27" t="s">
+      <c r="R37" s="21" t="s">
         <v>199</v>
       </c>
-      <c r="Q37" s="27" t="s">
+      <c r="S37" s="21" t="s">
         <v>194</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="O3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="Q3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="S3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
     <hyperlink ref="O4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="Q4" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="S4" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="O5" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="Q5" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="S5" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="O6" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="Q6" r:id="rId8" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="S6" r:id="rId8" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
     <hyperlink ref="O7" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="Q7" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="S7" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
     <hyperlink ref="O8" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="Q8" r:id="rId12" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="S8" r:id="rId12" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
     <hyperlink ref="O9" r:id="rId13" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="Q9" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="S9" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
     <hyperlink ref="O10" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="Q10" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="S10" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
     <hyperlink ref="O11" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="Q11" r:id="rId18" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="S11" r:id="rId18" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
     <hyperlink ref="O12" r:id="rId19" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="Q12" r:id="rId20" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="P15" r:id="rId21" xr:uid="{C440A0C4-B388-4CEB-BA5C-6198B15A0FDC}"/>
-    <hyperlink ref="P14" r:id="rId22" xr:uid="{630AA742-1285-4537-AFB4-BCA0666DA172}"/>
-    <hyperlink ref="P13" r:id="rId23" display="https://www.google.com/maps/place/Signature+By+M+Village+Beachfront+Hotel/@16.0809739,108.246656,19.74z/data=!4m9!3m8!1s0x3142171ddfd9fabd:0x79d9f6a4ee5545d!5m2!4m1!1i2!8m2!3d16.0811228!4d108.246958!16s%2Fg%2F11ydy3x0fc?entry=tts&amp;g_ep=EgoyMDI2MDUwMi4wIPu8ASoASAFQAw%3D%3D&amp;skid=d7f0fe9a-ad9f-4780-a71a-6b4b2a849114" xr:uid="{B926B33E-F12A-48D1-8511-6AB45751EBAD}"/>
-    <hyperlink ref="P17" r:id="rId24" display="https://www.google.com/maps/place/HN+Homes+-+Serviced+Apartment+CN2/@10.7958443,106.685193,20.14z/data=!4m6!3m5!1s0x317529ee4b3da91d:0xc4b5e37164766fcb!8m2!3d10.796192!4d106.6852857!16s%2Fg%2F11y5dzpc6q?entry=tts&amp;g_ep=EgoyMDI2MDUwMi4wIPu8ASoASAFQAw%3D%3D&amp;skid=93a8d717-382c-4a3f-8b58-4501ce2edc73" xr:uid="{9C6641CF-EBFC-4BA0-9093-F5709828908F}"/>
-    <hyperlink ref="P16" r:id="rId25" xr:uid="{69A9FD5A-8900-40CC-8650-1FD5666E1A90}"/>
-    <hyperlink ref="Q16" r:id="rId26" xr:uid="{A78542D9-54CA-45E4-A223-C3AE60A71AEC}"/>
-    <hyperlink ref="Q15" r:id="rId27" xr:uid="{34AA8874-BDB9-433C-894C-4086B3D10E18}"/>
-    <hyperlink ref="Q14" r:id="rId28" xr:uid="{C5EF6969-D170-4D45-B4D1-B63F6C5F637A}"/>
-    <hyperlink ref="Q13" r:id="rId29" xr:uid="{014AA80C-0CA0-4048-B788-6AADF95B469C}"/>
+    <hyperlink ref="S12" r:id="rId20" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="R15" r:id="rId21" xr:uid="{C440A0C4-B388-4CEB-BA5C-6198B15A0FDC}"/>
+    <hyperlink ref="R14" r:id="rId22" xr:uid="{630AA742-1285-4537-AFB4-BCA0666DA172}"/>
+    <hyperlink ref="R13" r:id="rId23" display="https://www.google.com/maps/place/Signature+By+M+Village+Beachfront+Hotel/@16.0809739,108.246656,19.74z/data=!4m9!3m8!1s0x3142171ddfd9fabd:0x79d9f6a4ee5545d!5m2!4m1!1i2!8m2!3d16.0811228!4d108.246958!16s%2Fg%2F11ydy3x0fc?entry=tts&amp;g_ep=EgoyMDI2MDUwMi4wIPu8ASoASAFQAw%3D%3D&amp;skid=d7f0fe9a-ad9f-4780-a71a-6b4b2a849114" xr:uid="{B926B33E-F12A-48D1-8511-6AB45751EBAD}"/>
+    <hyperlink ref="R17" r:id="rId24" display="https://www.google.com/maps/place/HN+Homes+-+Serviced+Apartment+CN2/@10.7958443,106.685193,20.14z/data=!4m6!3m5!1s0x317529ee4b3da91d:0xc4b5e37164766fcb!8m2!3d10.796192!4d106.6852857!16s%2Fg%2F11y5dzpc6q?entry=tts&amp;g_ep=EgoyMDI2MDUwMi4wIPu8ASoASAFQAw%3D%3D&amp;skid=93a8d717-382c-4a3f-8b58-4501ce2edc73" xr:uid="{9C6641CF-EBFC-4BA0-9093-F5709828908F}"/>
+    <hyperlink ref="R16" r:id="rId25" xr:uid="{69A9FD5A-8900-40CC-8650-1FD5666E1A90}"/>
+    <hyperlink ref="S16" r:id="rId26" xr:uid="{A78542D9-54CA-45E4-A223-C3AE60A71AEC}"/>
+    <hyperlink ref="S15" r:id="rId27" xr:uid="{34AA8874-BDB9-433C-894C-4086B3D10E18}"/>
+    <hyperlink ref="S14" r:id="rId28" xr:uid="{C5EF6969-D170-4D45-B4D1-B63F6C5F637A}"/>
+    <hyperlink ref="S13" r:id="rId29" xr:uid="{014AA80C-0CA0-4048-B788-6AADF95B469C}"/>
     <hyperlink ref="O13" r:id="rId30" xr:uid="{FAD10905-96EA-4FF4-8D3E-66716740EB52}"/>
     <hyperlink ref="O14" r:id="rId31" xr:uid="{741CA887-E15B-4987-8265-35B15215B779}"/>
     <hyperlink ref="O16" r:id="rId32" xr:uid="{514CBC1C-CE5A-4E1C-93FE-32FC429233CA}"/>
     <hyperlink ref="O15" r:id="rId33" xr:uid="{38B2A05A-F096-4641-A643-61EFD4404A6B}"/>
     <hyperlink ref="O17" r:id="rId34" xr:uid="{1696053E-D1FB-4156-945C-C980E10E68BF}"/>
-    <hyperlink ref="Q17" r:id="rId35" xr:uid="{F4651035-85EE-4C69-A618-11337D5578FD}"/>
-    <hyperlink ref="P4" r:id="rId36" xr:uid="{44258B57-2022-4512-8B2A-635A07EBD702}"/>
-    <hyperlink ref="P3" r:id="rId37" display="https://google.com/maps/place/Mercury+Beach+House/@16.0884991,108.2460601,17z/data=!4m10!3m9!1s0x314217f213c3031f:0xc3fa594a2c3558c1!5m2!4m1!1i2!8m2!3d16.0884991!4d108.248635!15sCjRNZXJjdXJ5IEJlYWNoIHdpdGggMkJScy0zIEJlZHMtUE9PTCAxMG0gdG8gdGhlIGJlYWNokgEFaG90ZWzgAQA!16s%2Fg%2F11jsp4x6y6?entry=tts&amp;g_ep=EgoyMDI2MDUwMi4wIPu8ASoASAFQAw%3D%3D&amp;skid=1ede066e-c2ca-421e-b8be-8fb412b82088" xr:uid="{5E649388-17BD-4B9E-A309-83F73D732E56}"/>
+    <hyperlink ref="S17" r:id="rId35" xr:uid="{F4651035-85EE-4C69-A618-11337D5578FD}"/>
+    <hyperlink ref="R4" r:id="rId36" xr:uid="{44258B57-2022-4512-8B2A-635A07EBD702}"/>
+    <hyperlink ref="R3" r:id="rId37" display="https://google.com/maps/place/Mercury+Beach+House/@16.0884991,108.2460601,17z/data=!4m10!3m9!1s0x314217f213c3031f:0xc3fa594a2c3558c1!5m2!4m1!1i2!8m2!3d16.0884991!4d108.248635!15sCjRNZXJjdXJ5IEJlYWNoIHdpdGggMkJScy0zIEJlZHMtUE9PTCAxMG0gdG8gdGhlIGJlYWNokgEFaG90ZWzgAQA!16s%2Fg%2F11jsp4x6y6?entry=tts&amp;g_ep=EgoyMDI2MDUwMi4wIPu8ASoASAFQAw%3D%3D&amp;skid=1ede066e-c2ca-421e-b8be-8fb412b82088" xr:uid="{5E649388-17BD-4B9E-A309-83F73D732E56}"/>
     <hyperlink ref="O18" r:id="rId38" xr:uid="{3091D75E-6088-4598-8E9F-AAED57F6C1BA}"/>
-    <hyperlink ref="Q18" r:id="rId39" xr:uid="{25F13F7C-12B6-437E-9A2B-B0DAF70F2289}"/>
-    <hyperlink ref="P18" r:id="rId40" xr:uid="{7C9ED5B5-E4F1-4017-B1AA-0ED1779D87A0}"/>
+    <hyperlink ref="S18" r:id="rId39" xr:uid="{25F13F7C-12B6-437E-9A2B-B0DAF70F2289}"/>
+    <hyperlink ref="R18" r:id="rId40" xr:uid="{7C9ED5B5-E4F1-4017-B1AA-0ED1779D87A0}"/>
     <hyperlink ref="O19" r:id="rId41" xr:uid="{02D47D6D-D06A-4E9B-89A3-1013A6528204}"/>
-    <hyperlink ref="Q19" r:id="rId42" xr:uid="{4058EB64-2805-4FB1-8891-6BE5ABA2BCF7}"/>
+    <hyperlink ref="S19" r:id="rId42" xr:uid="{4058EB64-2805-4FB1-8891-6BE5ABA2BCF7}"/>
     <hyperlink ref="O20" r:id="rId43" xr:uid="{E36242DA-FA92-435E-A4F4-5E09DBCC0459}"/>
-    <hyperlink ref="Q20" r:id="rId44" xr:uid="{1A85250B-E0EA-419A-8912-8E0070361A67}"/>
-    <hyperlink ref="P20" r:id="rId45" xr:uid="{BA88ECA5-3ED7-4453-9836-D0C2B7970406}"/>
+    <hyperlink ref="S20" r:id="rId44" xr:uid="{1A85250B-E0EA-419A-8912-8E0070361A67}"/>
+    <hyperlink ref="R20" r:id="rId45" xr:uid="{BA88ECA5-3ED7-4453-9836-D0C2B7970406}"/>
     <hyperlink ref="O21" r:id="rId46" xr:uid="{0DD9042B-7E82-4A1C-981B-95DC0F0E66E2}"/>
-    <hyperlink ref="Q21" r:id="rId47" xr:uid="{731BD421-991E-41A3-B362-526FFCECEF9A}"/>
-    <hyperlink ref="P21" r:id="rId48" xr:uid="{D7DB9A97-209E-4747-8DE8-F08B7B9C0EAD}"/>
+    <hyperlink ref="S21" r:id="rId47" xr:uid="{731BD421-991E-41A3-B362-526FFCECEF9A}"/>
+    <hyperlink ref="R21" r:id="rId48" xr:uid="{D7DB9A97-209E-4747-8DE8-F08B7B9C0EAD}"/>
     <hyperlink ref="O22" r:id="rId49" xr:uid="{12642672-35BC-482A-9371-0E5DB74F5099}"/>
-    <hyperlink ref="Q22" r:id="rId50" xr:uid="{A5C81D10-C165-437B-901D-AA3EFB878EA0}"/>
-    <hyperlink ref="P22" r:id="rId51" display="https://www.google.com/maps/place/The+Wooden+Page/@16.0816664,108.2334076,19.91z/data=!4m17!1m7!3m6!1s0x3142192ea7af17a7:0xc89a2c1fa256fb94!2zUXXDoW4gTeG6uSBLZW4!8m2!3d16.0822394!4d108.2332973!16s%2Fg%2F11ststlgnz!3m8!1s0x31421793e1758355:0x8ed7d69dd01fc78b!5m2!4m1!1i2!8m2!3d16.081863!4d108.2338518!16s%2Fg%2F11tn6kcvmm?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{EA20416F-B46B-4593-9C4F-4619361E8A40}"/>
-    <hyperlink ref="Q23" r:id="rId52" xr:uid="{0D44DED3-15A4-4C70-ACF1-835EC9CB0784}"/>
+    <hyperlink ref="S22" r:id="rId50" xr:uid="{A5C81D10-C165-437B-901D-AA3EFB878EA0}"/>
+    <hyperlink ref="R22" r:id="rId51" display="https://www.google.com/maps/place/The+Wooden+Page/@16.0816664,108.2334076,19.91z/data=!4m17!1m7!3m6!1s0x3142192ea7af17a7:0xc89a2c1fa256fb94!2zUXXDoW4gTeG6uSBLZW4!8m2!3d16.0822394!4d108.2332973!16s%2Fg%2F11ststlgnz!3m8!1s0x31421793e1758355:0x8ed7d69dd01fc78b!5m2!4m1!1i2!8m2!3d16.081863!4d108.2338518!16s%2Fg%2F11tn6kcvmm?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{EA20416F-B46B-4593-9C4F-4619361E8A40}"/>
+    <hyperlink ref="S23" r:id="rId52" xr:uid="{0D44DED3-15A4-4C70-ACF1-835EC9CB0784}"/>
     <hyperlink ref="O23" r:id="rId53" xr:uid="{17523106-EB31-4F77-B3B9-4E991D3D0404}"/>
-    <hyperlink ref="P23" r:id="rId54" xr:uid="{2EFFCD1F-C2FA-41DA-935E-DD5036698130}"/>
+    <hyperlink ref="R23" r:id="rId54" xr:uid="{2EFFCD1F-C2FA-41DA-935E-DD5036698130}"/>
     <hyperlink ref="O24" r:id="rId55" display="https://www.airbnb.com/rooms/1556187895484884653?adults=5&amp;check_in=2026-07-29&amp;check_out=2026-08-01&amp;search_mode=regular_search&amp;source_impression_id=p3_1778741985_P38laXBpbm4dgmkg&amp;previous_page_section_name=1000&amp;federated_search_id=eae37c30-5b51-4642-bae5-466b5db5b0ec" xr:uid="{E1B7FA9C-616E-4E02-896F-089B47A5A934}"/>
-    <hyperlink ref="Q24" r:id="rId56" xr:uid="{1E0BF4EE-7FD2-413A-B8BC-17F888B9350C}"/>
-    <hyperlink ref="P24" r:id="rId57" xr:uid="{E0FB3868-609E-4B43-84BD-F2563B94E8FE}"/>
+    <hyperlink ref="S24" r:id="rId56" xr:uid="{1E0BF4EE-7FD2-413A-B8BC-17F888B9350C}"/>
+    <hyperlink ref="R24" r:id="rId57" xr:uid="{E0FB3868-609E-4B43-84BD-F2563B94E8FE}"/>
     <hyperlink ref="O25" r:id="rId58" xr:uid="{9B5E18B5-8809-48EA-8F9C-9B2284647450}"/>
-    <hyperlink ref="Q25" r:id="rId59" xr:uid="{0C3F416E-D1C6-4038-900D-7FB07E51F560}"/>
-    <hyperlink ref="P25" r:id="rId60" display="https://www.google.com/maps/place/Pyramids+Restaurant+Halal+-+Middle+Eastern+Halal+Cuisine+%26+Arabic+Coffee+-+Ben+Thanh+Market+-+Tourists+in+Saigon+%7C+District+1/@10.7702105,106.7000776,20.36z/data=!4m9!1m2!2m1!1sle+chong+kie+ho+chi+minh!3m5!1s0x31752fcbafcb3c2b:0x71ce6a0be10dfbe0!8m2!3d10.7703643!4d106.7004126!16s%2Fg%2F11xflyz0cc?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{D022BFF9-C240-4D60-A3A0-B333C742D3C9}"/>
+    <hyperlink ref="S25" r:id="rId59" xr:uid="{0C3F416E-D1C6-4038-900D-7FB07E51F560}"/>
+    <hyperlink ref="R25" r:id="rId60" display="https://www.google.com/maps/place/Pyramids+Restaurant+Halal+-+Middle+Eastern+Halal+Cuisine+%26+Arabic+Coffee+-+Ben+Thanh+Market+-+Tourists+in+Saigon+%7C+District+1/@10.7702105,106.7000776,20.36z/data=!4m9!1m2!2m1!1sle+chong+kie+ho+chi+minh!3m5!1s0x31752fcbafcb3c2b:0x71ce6a0be10dfbe0!8m2!3d10.7703643!4d106.7004126!16s%2Fg%2F11xflyz0cc?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{D022BFF9-C240-4D60-A3A0-B333C742D3C9}"/>
     <hyperlink ref="O26" r:id="rId61" xr:uid="{29A8416D-BBCE-4236-BC58-637B32957D63}"/>
-    <hyperlink ref="Q26" r:id="rId62" xr:uid="{CD4A5948-5F18-4A06-86AC-0EF2FCEF752E}"/>
-    <hyperlink ref="P26" r:id="rId63" xr:uid="{75D88B4F-EB8E-4357-97C6-6EC93CCA55EB}"/>
-    <hyperlink ref="Q27" r:id="rId64" xr:uid="{D19B8FA7-95B8-4FF1-84CD-984128495F0A}"/>
+    <hyperlink ref="S26" r:id="rId62" xr:uid="{CD4A5948-5F18-4A06-86AC-0EF2FCEF752E}"/>
+    <hyperlink ref="R26" r:id="rId63" xr:uid="{75D88B4F-EB8E-4357-97C6-6EC93CCA55EB}"/>
+    <hyperlink ref="S27" r:id="rId64" xr:uid="{D19B8FA7-95B8-4FF1-84CD-984128495F0A}"/>
     <hyperlink ref="O27" r:id="rId65" xr:uid="{1E644DB5-138F-4514-87C1-8D01E021F60E}"/>
-    <hyperlink ref="P27" r:id="rId66" display="https://www.google.com/maps/place/121%2F49+L%C3%AA+Th%E1%BB%8B+Ri%C3%AAng,+B%E1%BA%BFn+Th%C3%A0nh,+H%E1%BB%93+Ch%C3%AD+Minh,+Vietnam/@10.7700643,106.69074,20.23z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3d0126385d:0x269ab3b058ed3698!8m2!3d10.770318!4d106.6908484!16s%2Fg%2F11j8h0qfj2?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{7834632D-5392-49B3-8759-ACE8294F0F5C}"/>
+    <hyperlink ref="R27" r:id="rId66" display="https://www.google.com/maps/place/121%2F49+L%C3%AA+Th%E1%BB%8B+Ri%C3%AAng,+B%E1%BA%BFn+Th%C3%A0nh,+H%E1%BB%93+Ch%C3%AD+Minh,+Vietnam/@10.7700643,106.69074,20.23z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3d0126385d:0x269ab3b058ed3698!8m2!3d10.770318!4d106.6908484!16s%2Fg%2F11j8h0qfj2?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{7834632D-5392-49B3-8759-ACE8294F0F5C}"/>
     <hyperlink ref="O28" r:id="rId67" xr:uid="{B47D79C9-7FA4-4084-8A7F-3496B862703D}"/>
-    <hyperlink ref="Q28" r:id="rId68" xr:uid="{0556A8F5-98BB-4842-A77C-819650662487}"/>
-    <hyperlink ref="P28" r:id="rId69" display="https://www.google.com/maps/place/C.Macro+Th%E1%BB%B1c+D%C6%B0%E1%BB%A1ng+S%E1%BA%A1ch+Vi%E1%BB%87t+Nam/@10.7639029,106.6927615,21z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752fb16bf8f9ad:0xa4de8d3544f2558a!8m2!3d10.7640143!4d106.692973!16s%2Fg%2F11g07s3lhd?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{DA4CD0AD-171C-4E4A-ADB4-C8467F04EA19}"/>
+    <hyperlink ref="S28" r:id="rId68" xr:uid="{0556A8F5-98BB-4842-A77C-819650662487}"/>
+    <hyperlink ref="R28" r:id="rId69" display="https://www.google.com/maps/place/C.Macro+Th%E1%BB%B1c+D%C6%B0%E1%BB%A1ng+S%E1%BA%A1ch+Vi%E1%BB%87t+Nam/@10.7639029,106.6927615,21z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752fb16bf8f9ad:0xa4de8d3544f2558a!8m2!3d10.7640143!4d106.692973!16s%2Fg%2F11g07s3lhd?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{DA4CD0AD-171C-4E4A-ADB4-C8467F04EA19}"/>
     <hyperlink ref="O29" r:id="rId70" xr:uid="{A201A6E0-4C43-489F-B008-F6087D50353A}"/>
-    <hyperlink ref="Q29" r:id="rId71" xr:uid="{4D02F78F-8922-4FAC-B501-69FD9E985CA3}"/>
-    <hyperlink ref="P29" r:id="rId72" display="https://www.google.com/maps/place/229+Pham+Ngu+Lao/@10.767733,106.6914827,18.95z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3df2e2bc1b:0xf5b67606e28b5f25!8m2!3d10.7682962!4d106.6926399!16s%2Fg%2F11z5nct8zk?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{D4453A9F-7434-43C4-91D7-143D85457C23}"/>
-    <hyperlink ref="P33" r:id="rId73" display="https://www.google.com/maps/place/Signy+House+Hotel+%26+Apartments+-+15B+Tr%E1%BA%A7n+Kh%C3%A1nh+D%C6%B0/@10.7937942,106.6782041,15z/data=!4m9!3m8!1s0x3175297257c4b02d:0xf2b70587ed8538c2!5m2!4m1!1i2!8m2!3d10.7937733!4d106.6884824!16s%2Fg%2F11fkgscnkj?entry=tts&amp;g_ep=EgoyMDI2MDUxMy4wIPu8ASoASAFQAw%3D%3D&amp;skid=47be7804-7c50-4e29-9594-7f7d7e9438b4" xr:uid="{D5F0658E-83F9-4842-8E1B-C884A47FB73D}"/>
-    <hyperlink ref="Q33" r:id="rId74" xr:uid="{1A8C3643-1642-451E-9410-6CF9FFEC2D94}"/>
-    <hyperlink ref="Q34" r:id="rId75" xr:uid="{C53609F4-15E7-4443-B02F-0C74133BB825}"/>
+    <hyperlink ref="S29" r:id="rId71" xr:uid="{4D02F78F-8922-4FAC-B501-69FD9E985CA3}"/>
+    <hyperlink ref="R29" r:id="rId72" display="https://www.google.com/maps/place/229+Pham+Ngu+Lao/@10.767733,106.6914827,18.95z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3df2e2bc1b:0xf5b67606e28b5f25!8m2!3d10.7682962!4d106.6926399!16s%2Fg%2F11z5nct8zk?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{D4453A9F-7434-43C4-91D7-143D85457C23}"/>
+    <hyperlink ref="R33" r:id="rId73" display="https://www.google.com/maps/place/Signy+House+Hotel+%26+Apartments+-+15B+Tr%E1%BA%A7n+Kh%C3%A1nh+D%C6%B0/@10.7937942,106.6782041,15z/data=!4m9!3m8!1s0x3175297257c4b02d:0xf2b70587ed8538c2!5m2!4m1!1i2!8m2!3d10.7937733!4d106.6884824!16s%2Fg%2F11fkgscnkj?entry=tts&amp;g_ep=EgoyMDI2MDUxMy4wIPu8ASoASAFQAw%3D%3D&amp;skid=47be7804-7c50-4e29-9594-7f7d7e9438b4" xr:uid="{D5F0658E-83F9-4842-8E1B-C884A47FB73D}"/>
+    <hyperlink ref="S33" r:id="rId74" xr:uid="{1A8C3643-1642-451E-9410-6CF9FFEC2D94}"/>
+    <hyperlink ref="S34" r:id="rId75" xr:uid="{C53609F4-15E7-4443-B02F-0C74133BB825}"/>
     <hyperlink ref="O34" r:id="rId76" xr:uid="{3AC6E81A-6881-4337-8506-B3D382C7CF17}"/>
-    <hyperlink ref="P34" r:id="rId77" xr:uid="{687A6D4C-311E-495B-B859-7DC574CC4A73}"/>
+    <hyperlink ref="R34" r:id="rId77" xr:uid="{687A6D4C-311E-495B-B859-7DC574CC4A73}"/>
     <hyperlink ref="O35" r:id="rId78" xr:uid="{1FA4B93F-03BC-48A9-8B51-50064FF7FE02}"/>
-    <hyperlink ref="Q35" r:id="rId79" xr:uid="{A5F8DC54-E881-4FCB-9159-36AD18BF83BA}"/>
-    <hyperlink ref="P35" r:id="rId80" xr:uid="{A32DF229-EDA9-4BC6-ADE4-599B1CA01F6B}"/>
+    <hyperlink ref="S35" r:id="rId79" xr:uid="{A5F8DC54-E881-4FCB-9159-36AD18BF83BA}"/>
+    <hyperlink ref="R35" r:id="rId80" xr:uid="{A32DF229-EDA9-4BC6-ADE4-599B1CA01F6B}"/>
     <hyperlink ref="O36" r:id="rId81" xr:uid="{E550138A-19A3-4433-933A-9E1E3665AFD8}"/>
-    <hyperlink ref="Q36" r:id="rId82" xr:uid="{DE0FF8BC-6382-4390-8FFB-A33701AE1678}"/>
-    <hyperlink ref="P36" r:id="rId83" display="https://maps.app.goo.gl/BoXEQmtD7p7UBWQF9" xr:uid="{3E71EB02-0A48-463C-BD49-37B122A1E55C}"/>
+    <hyperlink ref="S36" r:id="rId82" xr:uid="{DE0FF8BC-6382-4390-8FFB-A33701AE1678}"/>
+    <hyperlink ref="R36" r:id="rId83" display="https://maps.app.goo.gl/BoXEQmtD7p7UBWQF9" xr:uid="{3E71EB02-0A48-463C-BD49-37B122A1E55C}"/>
     <hyperlink ref="O37" r:id="rId84" xr:uid="{83E719A9-EBF2-4255-8E50-F1AFDD3DEB65}"/>
-    <hyperlink ref="Q37" r:id="rId85" xr:uid="{049758F8-0E93-4846-AF70-5FFC65C94ABA}"/>
-    <hyperlink ref="P37" r:id="rId86" display="https://maps.app.goo.gl/8CGQz8X495XTkWsG6" xr:uid="{7628EC14-1A53-4FF5-94FD-C8B5E44766D9}"/>
-    <hyperlink ref="O30" r:id="rId87" xr:uid="{50B44A8F-1E12-43F2-8CE1-88FBDBCB2862}"/>
-    <hyperlink ref="O31" r:id="rId88" xr:uid="{E6A06F26-4042-4F78-98CB-A4703A09D563}"/>
-    <hyperlink ref="O32" r:id="rId89" xr:uid="{BB03F22A-3802-4705-A436-312DA30713C2}"/>
-    <hyperlink ref="Q30" r:id="rId90" xr:uid="{BE32A7B1-BB98-49B1-B4DF-3E2676C5EAAD}"/>
-    <hyperlink ref="P30" r:id="rId91" display="https://www.google.com/maps/place/C%C4%83n+H%E1%BB%99+Lavida+Plus+Qu%E1%BA%ADn+7/@10.7271647,106.6994728,16.77z/data=!4m6!3m5!1s0x31752ffb91d6c583:0xa398b70b12abf8dd!8m2!3d10.7272695!4d106.7018208!16s%2Fg%2F11m5y0434z?entry=ttu&amp;g_ep=EgoyMDI2MDUxMy4wIKXMDSoASAFQAw%3D%3D" xr:uid="{C367F6F5-5149-41FF-934E-A36B4A5B4344}"/>
-    <hyperlink ref="Q31" r:id="rId92" xr:uid="{F0DAF66C-579C-42A1-B3A3-563254C38222}"/>
-    <hyperlink ref="P31" r:id="rId93" display="https://www.google.com/maps/place/H%E1%BB%93ng+Tr%C3%A0+Ng%C3%B4+Gia+H078/@10.7636066,106.6951405,20z/data=!4m6!3m5!1s0x31752fb67d1f4b5f:0x4cc87f858721ebe3!8m2!3d10.763715!4d106.69538!16s%2Fg%2F11t0rz2fvv?entry=ttu&amp;g_ep=EgoyMDI2MDUxMy4wIKXMDSoASAFQAw%3D%3D" xr:uid="{4F1ED331-255E-45A6-B8C3-572C0191A949}"/>
-    <hyperlink ref="Q32" r:id="rId94" xr:uid="{50750A5D-2EAE-413E-9D75-3C11EC2D65F6}"/>
+    <hyperlink ref="S37" r:id="rId85" xr:uid="{049758F8-0E93-4846-AF70-5FFC65C94ABA}"/>
+    <hyperlink ref="R37" r:id="rId86" display="https://maps.app.goo.gl/8CGQz8X495XTkWsG6" xr:uid="{7628EC14-1A53-4FF5-94FD-C8B5E44766D9}"/>
+    <hyperlink ref="Q30" r:id="rId87" xr:uid="{50B44A8F-1E12-43F2-8CE1-88FBDBCB2862}"/>
+    <hyperlink ref="Q31" r:id="rId88" xr:uid="{E6A06F26-4042-4F78-98CB-A4703A09D563}"/>
+    <hyperlink ref="Q32" r:id="rId89" xr:uid="{BB03F22A-3802-4705-A436-312DA30713C2}"/>
+    <hyperlink ref="S30" r:id="rId90" xr:uid="{BE32A7B1-BB98-49B1-B4DF-3E2676C5EAAD}"/>
+    <hyperlink ref="R30" r:id="rId91" display="https://www.google.com/maps/place/C%C4%83n+H%E1%BB%99+Lavida+Plus+Qu%E1%BA%ADn+7/@10.7271647,106.6994728,16.77z/data=!4m6!3m5!1s0x31752ffb91d6c583:0xa398b70b12abf8dd!8m2!3d10.7272695!4d106.7018208!16s%2Fg%2F11m5y0434z?entry=ttu&amp;g_ep=EgoyMDI2MDUxMy4wIKXMDSoASAFQAw%3D%3D" xr:uid="{C367F6F5-5149-41FF-934E-A36B4A5B4344}"/>
+    <hyperlink ref="S31" r:id="rId92" xr:uid="{F0DAF66C-579C-42A1-B3A3-563254C38222}"/>
+    <hyperlink ref="R31" r:id="rId93" display="https://www.google.com/maps/place/H%E1%BB%93ng+Tr%C3%A0+Ng%C3%B4+Gia+H078/@10.7636066,106.6951405,20z/data=!4m6!3m5!1s0x31752fb67d1f4b5f:0x4cc87f858721ebe3!8m2!3d10.763715!4d106.69538!16s%2Fg%2F11t0rz2fvv?entry=ttu&amp;g_ep=EgoyMDI2MDUxMy4wIKXMDSoASAFQAw%3D%3D" xr:uid="{4F1ED331-255E-45A6-B8C3-572C0191A949}"/>
+    <hyperlink ref="S32" r:id="rId94" xr:uid="{50750A5D-2EAE-413E-9D75-3C11EC2D65F6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>